<commit_message>
Add Front Squat as a standard
New lower_strength lift (orm, ×bodyweight), scored beside Back Squat and
Deadlift. Tiers seeded at ~0.82× back squat (M 1.05/1.35/1.65/2.05,
F 0.80/1.05/1.30/1.65) — coach-curated ratio, flagged beta like the rest.

Added to the Excel master (Benchmarks_Sourcing + Standards via seed),
regenerated the lift config, gave it an explicit "Front Squat" label,
and generated its /standards/front-squat/ SEO page.

Verified in Chrome: appears in the entry grid; 43 SEO pages; 105 tests pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -480,7 +480,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -717,7 +717,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>deadlift_1rm</v>
+        <v>front_squat_1rm</v>
       </c>
       <c r="B8" t="str">
         <v>lower_strength</v>
@@ -735,30 +735,30 @@
         <v>bodyweight</v>
       </c>
       <c r="G8" t="str">
-        <v>OpenPowerlifting</v>
+        <v>Coaching ratios</v>
       </c>
       <c r="H8" t="str">
-        <v>CC0 / public domain</v>
+        <v>n/a</v>
       </c>
       <c r="I8" t="str">
-        <v>Yes (no restriction)</v>
+        <v>Yes</v>
       </c>
       <c r="J8" t="str">
-        <v>Competitive lifters</v>
+        <v>Trained adults</v>
       </c>
       <c r="K8" t="str">
-        <v>Licensed data (adjust)</v>
+        <v>Coach-curated (~0.82x back squat)</v>
       </c>
       <c r="L8" t="str">
-        <v>Contested in PL</v>
+        <v>Front squat 1RM</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>bench_1rm</v>
+        <v>deadlift_1rm</v>
       </c>
       <c r="B9" t="str">
-        <v>upper_strength</v>
+        <v>lower_strength</v>
       </c>
       <c r="C9" t="str">
         <v>orm</v>
@@ -788,12 +788,12 @@
         <v>Licensed data (adjust)</v>
       </c>
       <c r="L9" t="str">
-        <v>Bench contested in PL</v>
+        <v>Contested in PL</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>strict_press_1rm</v>
+        <v>bench_1rm</v>
       </c>
       <c r="B10" t="str">
         <v>upper_strength</v>
@@ -811,30 +811,30 @@
         <v>bodyweight</v>
       </c>
       <c r="G10" t="str">
-        <v>Expert-curated (not a contested lift)</v>
+        <v>OpenPowerlifting</v>
       </c>
       <c r="H10" t="str">
-        <v>None</v>
+        <v>CC0 / public domain</v>
       </c>
       <c r="I10" t="str">
-        <v>Expert</v>
+        <v>Yes (no restriction)</v>
       </c>
       <c r="J10" t="str">
-        <v>Own users</v>
+        <v>Competitive lifters</v>
       </c>
       <c r="K10" t="str">
-        <v>Expert-curated + own-data</v>
+        <v>Licensed data (adjust)</v>
       </c>
       <c r="L10" t="str">
-        <v>Anchor ratio vs bench / bodyweight; refine from own data</v>
+        <v>Bench contested in PL</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>snatch_1rm</v>
+        <v>strict_press_1rm</v>
       </c>
       <c r="B11" t="str">
-        <v>olympic</v>
+        <v>upper_strength</v>
       </c>
       <c r="C11" t="str">
         <v>orm</v>
@@ -849,27 +849,27 @@
         <v>bodyweight</v>
       </c>
       <c r="G11" t="str">
-        <v>IWF comp data (elite) + coaching ratios</v>
+        <v>Expert-curated (not a contested lift)</v>
       </c>
       <c r="H11" t="str">
-        <v>Proprietary / unclear</v>
+        <v>None</v>
       </c>
       <c r="I11" t="str">
-        <v>License required / expert</v>
+        <v>Expert</v>
       </c>
       <c r="J11" t="str">
-        <v>Elite weightlifters</v>
+        <v>Own users</v>
       </c>
       <c r="K11" t="str">
         <v>Expert-curated + own-data</v>
       </c>
       <c r="L11" t="str">
-        <v>Comp data elite-biased; anchor with coaching ratios</v>
+        <v>Anchor ratio vs bench / bodyweight; refine from own data</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>clean_jerk_1rm</v>
+        <v>snatch_1rm</v>
       </c>
       <c r="B12" t="str">
         <v>olympic</v>
@@ -887,7 +887,7 @@
         <v>bodyweight</v>
       </c>
       <c r="G12" t="str">
-        <v>IWF comp data + coaching ratios</v>
+        <v>IWF comp data (elite) + coaching ratios</v>
       </c>
       <c r="H12" t="str">
         <v>Proprietary / unclear</v>
@@ -902,15 +902,15 @@
         <v>Expert-curated + own-data</v>
       </c>
       <c r="L12" t="str">
-        <v>As snatch</v>
+        <v>Comp data elite-biased; anchor with coaching ratios</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>power_clean_1rm</v>
+        <v>clean_jerk_1rm</v>
       </c>
       <c r="B13" t="str">
-        <v>power</v>
+        <v>olympic</v>
       </c>
       <c r="C13" t="str">
         <v>orm</v>
@@ -925,74 +925,74 @@
         <v>bodyweight</v>
       </c>
       <c r="G13" t="str">
-        <v>Expert-curated (not contested)</v>
+        <v>IWF comp data + coaching ratios</v>
       </c>
       <c r="H13" t="str">
-        <v>None</v>
+        <v>Proprietary / unclear</v>
       </c>
       <c r="I13" t="str">
-        <v>Expert</v>
+        <v>License required / expert</v>
       </c>
       <c r="J13" t="str">
-        <v>Own users</v>
+        <v>Elite weightlifters</v>
       </c>
       <c r="K13" t="str">
         <v>Expert-curated + own-data</v>
       </c>
       <c r="L13" t="str">
-        <v>Ratio vs clean &amp; jerk; refine from own data</v>
+        <v>As snatch</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>broad_jump</v>
+        <v>power_clean_1rm</v>
       </c>
       <c r="B14" t="str">
         <v>power</v>
       </c>
       <c r="C14" t="str">
-        <v>manual</v>
+        <v>orm</v>
       </c>
       <c r="D14" t="str">
-        <v>cm</v>
+        <v>xBW</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
       </c>
       <c r="F14" t="str">
-        <v>absolute</v>
+        <v>bodyweight</v>
       </c>
       <c r="G14" t="str">
-        <v>Athletic / combine normative data + expert</v>
+        <v>Expert-curated (not contested)</v>
       </c>
       <c r="H14" t="str">
-        <v>Mixed / public norms</v>
+        <v>None</v>
       </c>
       <c r="I14" t="str">
-        <v>Check per source</v>
+        <v>Expert</v>
       </c>
       <c r="J14" t="str">
-        <v>Athletic test populations</v>
+        <v>Own users</v>
       </c>
       <c r="K14" t="str">
-        <v>Published norms + own-data</v>
+        <v>Expert-curated + own-data</v>
       </c>
       <c r="L14" t="str">
-        <v>Sex-split absolute distance</v>
+        <v>Ratio vs clean &amp; jerk; refine from own data</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>strict_pullups</v>
+        <v>broad_jump</v>
       </c>
       <c r="B15" t="str">
-        <v>gymnastics</v>
+        <v>power</v>
       </c>
       <c r="C15" t="str">
         <v>manual</v>
       </c>
       <c r="D15" t="str">
-        <v>reps</v>
+        <v>cm</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -1001,27 +1001,27 @@
         <v>absolute</v>
       </c>
       <c r="G15" t="str">
-        <v>Expert-curated (no public dataset)</v>
+        <v>Athletic / combine normative data + expert</v>
       </c>
       <c r="H15" t="str">
-        <v>None</v>
+        <v>Mixed / public norms</v>
       </c>
       <c r="I15" t="str">
-        <v>Expert</v>
+        <v>Check per source</v>
       </c>
       <c r="J15" t="str">
-        <v>Own users</v>
+        <v>Athletic test populations</v>
       </c>
       <c r="K15" t="str">
-        <v>Expert-curated + own-data</v>
+        <v>Published norms + own-data</v>
       </c>
       <c r="L15" t="str">
-        <v>Recalibrate from own data quickly</v>
+        <v>Sex-split absolute distance</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>hspu</v>
+        <v>strict_pullups</v>
       </c>
       <c r="B16" t="str">
         <v>gymnastics</v>
@@ -1039,7 +1039,7 @@
         <v>absolute</v>
       </c>
       <c r="G16" t="str">
-        <v>Expert-curated</v>
+        <v>Expert-curated (no public dataset)</v>
       </c>
       <c r="H16" t="str">
         <v>None</v>
@@ -1054,12 +1054,12 @@
         <v>Expert-curated + own-data</v>
       </c>
       <c r="L16" t="str">
-        <v>Define Rx standard (kipping vs strict) explicitly</v>
+        <v>Recalibrate from own data quickly</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>t2b</v>
+        <v>hspu</v>
       </c>
       <c r="B17" t="str">
         <v>gymnastics</v>
@@ -1091,10 +1091,13 @@
       <c r="K17" t="str">
         <v>Expert-curated + own-data</v>
       </c>
+      <c r="L17" t="str">
+        <v>Strict HSPU — head to floor, no kip, full lockout</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>du_unbroken</v>
+        <v>t2b</v>
       </c>
       <c r="B18" t="str">
         <v>gymnastics</v>
@@ -1126,13 +1129,10 @@
       <c r="K18" t="str">
         <v>Expert-curated + own-data</v>
       </c>
-      <c r="L18" t="str">
-        <v>Unbroken double-unders</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>max_mu</v>
+        <v>du_unbroken</v>
       </c>
       <c r="B19" t="str">
         <v>gymnastics</v>
@@ -1165,21 +1165,21 @@
         <v>Expert-curated + own-data</v>
       </c>
       <c r="L19" t="str">
-        <v>Bar or ring — specify</v>
+        <v>Unbroken double-unders</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>plank_hold</v>
+        <v>max_mu</v>
       </c>
       <c r="B20" t="str">
-        <v>core_endurance</v>
+        <v>gymnastics</v>
       </c>
       <c r="C20" t="str">
         <v>manual</v>
       </c>
       <c r="D20" t="str">
-        <v>mm:ss</v>
+        <v>reps</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -1188,10 +1188,10 @@
         <v>absolute</v>
       </c>
       <c r="G20" t="str">
-        <v>Normative fitness data + expert</v>
+        <v>Expert-curated</v>
       </c>
       <c r="H20" t="str">
-        <v>Mixed</v>
+        <v>None</v>
       </c>
       <c r="I20" t="str">
         <v>Expert</v>
@@ -1203,15 +1203,15 @@
         <v>Expert-curated + own-data</v>
       </c>
       <c r="L20" t="str">
-        <v>Longer = better (higher_is_better)</v>
+        <v>Bar or ring — specify</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>grip_deadhang</v>
+        <v>plank_hold</v>
       </c>
       <c r="B21" t="str">
-        <v>grip (optional)</v>
+        <v>core_endurance</v>
       </c>
       <c r="C21" t="str">
         <v>manual</v>
@@ -1226,10 +1226,10 @@
         <v>absolute</v>
       </c>
       <c r="G21" t="str">
-        <v>Expert-curated</v>
+        <v>Normative fitness data + expert</v>
       </c>
       <c r="H21" t="str">
-        <v>None</v>
+        <v>Mixed</v>
       </c>
       <c r="I21" t="str">
         <v>Expert</v>
@@ -1238,36 +1238,36 @@
         <v>Own users</v>
       </c>
       <c r="K21" t="str">
-        <v>Optional — off by default</v>
+        <v>Expert-curated + own-data</v>
       </c>
       <c r="L21" t="str">
-        <v>Carry-over from ORS</v>
+        <v>Longer = better (higher_is_better)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ruck_time</v>
+        <v>grip_deadhang</v>
       </c>
       <c r="B22" t="str">
-        <v>rucking (optional)</v>
+        <v>grip (optional)</v>
       </c>
       <c r="C22" t="str">
-        <v>race_times</v>
+        <v>manual</v>
       </c>
       <c r="D22" t="str">
         <v>mm:ss</v>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="str">
         <v>absolute</v>
       </c>
       <c r="G22" t="str">
-        <v>Expert / military standards</v>
+        <v>Expert-curated</v>
       </c>
       <c r="H22" t="str">
-        <v>Mixed</v>
+        <v>None</v>
       </c>
       <c r="I22" t="str">
         <v>Expert</v>
@@ -1282,17 +1282,54 @@
         <v>Carry-over from ORS</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>ruck_time</v>
+      </c>
+      <c r="B23" t="str">
+        <v>rucking (optional)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>race_times</v>
+      </c>
+      <c r="D23" t="str">
+        <v>mm:ss</v>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" t="str">
+        <v>absolute</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Expert / military standards</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Expert</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Own users</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Optional — off by default</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Carry-over from ORS</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1653,7 +1690,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>deadlift_1rm</v>
+        <v>front_squat_1rm</v>
       </c>
       <c r="B13" t="str">
         <v>M</v>
@@ -1665,19 +1702,19 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>1.5</v>
+        <v>1.05</v>
       </c>
       <c r="F13">
-        <v>1.9</v>
+        <v>1.35</v>
       </c>
       <c r="G13">
-        <v>2.3</v>
+        <v>1.65</v>
       </c>
       <c r="H13">
-        <v>2.8</v>
+        <v>2.05</v>
       </c>
       <c r="I13" t="str">
-        <v>OpenPowerlifting (adj.)</v>
+        <v>Coaching ratios (≈0.82× back squat)</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -1685,7 +1722,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>deadlift_1rm</v>
+        <v>front_squat_1rm</v>
       </c>
       <c r="B14" t="str">
         <v>F</v>
@@ -1697,19 +1734,19 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="F14">
-        <v>1.5</v>
+        <v>1.05</v>
       </c>
       <c r="G14">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="H14">
-        <v>2.4</v>
+        <v>1.65</v>
       </c>
       <c r="I14" t="str">
-        <v>OpenPowerlifting (adj.)</v>
+        <v>Coaching ratios (≈0.82× back squat)</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -1717,7 +1754,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>bench_1rm</v>
+        <v>deadlift_1rm</v>
       </c>
       <c r="B15" t="str">
         <v>M</v>
@@ -1729,16 +1766,16 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F15">
-        <v>1.25</v>
+        <v>1.9</v>
       </c>
       <c r="G15">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="I15" t="str">
         <v>OpenPowerlifting (adj.)</v>
@@ -1749,7 +1786,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>bench_1rm</v>
+        <v>deadlift_1rm</v>
       </c>
       <c r="B16" t="str">
         <v>F</v>
@@ -1761,16 +1798,16 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F16">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="H16">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="I16" t="str">
         <v>OpenPowerlifting (adj.)</v>
@@ -1781,7 +1818,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>strict_press_1rm</v>
+        <v>bench_1rm</v>
       </c>
       <c r="B17" t="str">
         <v>M</v>
@@ -1793,19 +1830,19 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>0.8</v>
+        <v>1.25</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="H17">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="I17" t="str">
-        <v>Expert-curated</v>
+        <v>OpenPowerlifting (adj.)</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -1813,7 +1850,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>strict_press_1rm</v>
+        <v>bench_1rm</v>
       </c>
       <c r="B18" t="str">
         <v>F</v>
@@ -1825,19 +1862,19 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="F18">
-        <v>0.55</v>
+        <v>0.8</v>
       </c>
       <c r="G18">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="I18" t="str">
-        <v>Expert-curated</v>
+        <v>OpenPowerlifting (adj.)</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -1845,7 +1882,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>snatch_1rm</v>
+        <v>strict_press_1rm</v>
       </c>
       <c r="B19" t="str">
         <v>M</v>
@@ -1857,19 +1894,19 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F19">
-        <v>0.95</v>
+        <v>0.8</v>
       </c>
       <c r="G19">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H19">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="I19" t="str">
-        <v>Expert + coaching ratios</v>
+        <v>Expert-curated</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1877,7 +1914,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>snatch_1rm</v>
+        <v>strict_press_1rm</v>
       </c>
       <c r="B20" t="str">
         <v>F</v>
@@ -1889,19 +1926,19 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F20">
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="G20">
-        <v>0.85</v>
+        <v>0.7</v>
       </c>
       <c r="H20">
-        <v>1.05</v>
+        <v>0.9</v>
       </c>
       <c r="I20" t="str">
-        <v>Expert + coaching ratios</v>
+        <v>Expert-curated</v>
       </c>
       <c r="J20" t="str">
         <v/>
@@ -1909,7 +1946,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>clean_jerk_1rm</v>
+        <v>snatch_1rm</v>
       </c>
       <c r="B21" t="str">
         <v>M</v>
@@ -1921,16 +1958,16 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="F21">
+        <v>0.95</v>
+      </c>
+      <c r="G21">
         <v>1.2</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>1.5</v>
-      </c>
-      <c r="H21">
-        <v>1.85</v>
       </c>
       <c r="I21" t="str">
         <v>Expert + coaching ratios</v>
@@ -1941,7 +1978,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>clean_jerk_1rm</v>
+        <v>snatch_1rm</v>
       </c>
       <c r="B22" t="str">
         <v>F</v>
@@ -1953,16 +1990,16 @@
         <v>0</v>
       </c>
       <c r="E22">
+        <v>0.5</v>
+      </c>
+      <c r="F22">
         <v>0.65</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>0.85</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>1.05</v>
-      </c>
-      <c r="H22">
-        <v>1.3</v>
       </c>
       <c r="I22" t="str">
         <v>Expert + coaching ratios</v>
@@ -1973,7 +2010,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>power_clean_1rm</v>
+        <v>clean_jerk_1rm</v>
       </c>
       <c r="B23" t="str">
         <v>M</v>
@@ -1985,19 +2022,19 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="F23">
-        <v>1.05</v>
+        <v>1.2</v>
       </c>
       <c r="G23">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="H23">
-        <v>1.6</v>
+        <v>1.85</v>
       </c>
       <c r="I23" t="str">
-        <v>Expert-curated</v>
+        <v>Expert + coaching ratios</v>
       </c>
       <c r="J23" t="str">
         <v/>
@@ -2005,7 +2042,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>power_clean_1rm</v>
+        <v>clean_jerk_1rm</v>
       </c>
       <c r="B24" t="str">
         <v>F</v>
@@ -2017,19 +2054,19 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="F24">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="G24">
-        <v>0.95</v>
+        <v>1.05</v>
       </c>
       <c r="H24">
-        <v>1.15</v>
+        <v>1.3</v>
       </c>
       <c r="I24" t="str">
-        <v>Expert-curated</v>
+        <v>Expert + coaching ratios</v>
       </c>
       <c r="J24" t="str">
         <v/>
@@ -2037,31 +2074,31 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>broad_jump</v>
+        <v>power_clean_1rm</v>
       </c>
       <c r="B25" t="str">
         <v>M</v>
       </c>
       <c r="C25" t="str">
-        <v>cm</v>
+        <v>xBW</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
       <c r="E25">
-        <v>200</v>
+        <v>0.8</v>
       </c>
       <c r="F25">
-        <v>230</v>
+        <v>1.05</v>
       </c>
       <c r="G25">
-        <v>260</v>
+        <v>1.3</v>
       </c>
       <c r="H25">
-        <v>300</v>
+        <v>1.6</v>
       </c>
       <c r="I25" t="str">
-        <v>Combine norms + expert</v>
+        <v>Expert-curated</v>
       </c>
       <c r="J25" t="str">
         <v/>
@@ -2069,31 +2106,31 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>broad_jump</v>
+        <v>power_clean_1rm</v>
       </c>
       <c r="B26" t="str">
         <v>F</v>
       </c>
       <c r="C26" t="str">
-        <v>cm</v>
+        <v>xBW</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
       <c r="E26">
-        <v>160</v>
+        <v>0.55</v>
       </c>
       <c r="F26">
-        <v>185</v>
+        <v>0.75</v>
       </c>
       <c r="G26">
-        <v>210</v>
+        <v>0.95</v>
       </c>
       <c r="H26">
-        <v>245</v>
+        <v>1.15</v>
       </c>
       <c r="I26" t="str">
-        <v>Combine norms + expert</v>
+        <v>Expert-curated</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -2101,31 +2138,31 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>strict_pullups</v>
+        <v>broad_jump</v>
       </c>
       <c r="B27" t="str">
         <v>M</v>
       </c>
       <c r="C27" t="str">
-        <v>reps</v>
+        <v>cm</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
       <c r="E27">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="F27">
-        <v>11</v>
+        <v>230</v>
       </c>
       <c r="G27">
-        <v>18</v>
+        <v>260</v>
       </c>
       <c r="H27">
-        <v>28</v>
+        <v>300</v>
       </c>
       <c r="I27" t="str">
-        <v>Expert-curated</v>
+        <v>Combine norms + expert</v>
       </c>
       <c r="J27" t="str">
         <v/>
@@ -2133,31 +2170,31 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>strict_pullups</v>
+        <v>broad_jump</v>
       </c>
       <c r="B28" t="str">
         <v>F</v>
       </c>
       <c r="C28" t="str">
-        <v>reps</v>
+        <v>cm</v>
       </c>
       <c r="D28">
         <v>0</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>160</v>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>185</v>
       </c>
       <c r="G28">
-        <v>10</v>
+        <v>210</v>
       </c>
       <c r="H28">
-        <v>18</v>
+        <v>245</v>
       </c>
       <c r="I28" t="str">
-        <v>Expert-curated</v>
+        <v>Combine norms + expert</v>
       </c>
       <c r="J28" t="str">
         <v/>
@@ -2165,7 +2202,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>hspu</v>
+        <v>strict_pullups</v>
       </c>
       <c r="B29" t="str">
         <v>M</v>
@@ -2177,16 +2214,16 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F29">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G29">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H29">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I29" t="str">
         <v>Expert-curated</v>
@@ -2197,7 +2234,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>hspu</v>
+        <v>strict_pullups</v>
       </c>
       <c r="B30" t="str">
         <v>F</v>
@@ -2212,13 +2249,13 @@
         <v>1</v>
       </c>
       <c r="F30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G30">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H30">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I30" t="str">
         <v>Expert-curated</v>
@@ -2229,7 +2266,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>t2b</v>
+        <v>hspu</v>
       </c>
       <c r="B31" t="str">
         <v>M</v>
@@ -2241,16 +2278,16 @@
         <v>0</v>
       </c>
       <c r="E31">
+        <v>3</v>
+      </c>
+      <c r="F31">
         <v>8</v>
       </c>
-      <c r="F31">
-        <v>18</v>
-      </c>
       <c r="G31">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H31">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I31" t="str">
         <v>Expert-curated</v>
@@ -2261,7 +2298,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>t2b</v>
+        <v>hspu</v>
       </c>
       <c r="B32" t="str">
         <v>F</v>
@@ -2273,16 +2310,16 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F32">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G32">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="H32">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="I32" t="str">
         <v>Expert-curated</v>
@@ -2293,7 +2330,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>du_unbroken</v>
+        <v>t2b</v>
       </c>
       <c r="B33" t="str">
         <v>M</v>
@@ -2305,16 +2342,16 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F33">
+        <v>18</v>
+      </c>
+      <c r="G33">
+        <v>30</v>
+      </c>
+      <c r="H33">
         <v>50</v>
-      </c>
-      <c r="G33">
-        <v>100</v>
-      </c>
-      <c r="H33">
-        <v>200</v>
       </c>
       <c r="I33" t="str">
         <v>Expert-curated</v>
@@ -2325,7 +2362,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>du_unbroken</v>
+        <v>t2b</v>
       </c>
       <c r="B34" t="str">
         <v>F</v>
@@ -2337,16 +2374,16 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F34">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="G34">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="H34">
-        <v>180</v>
+        <v>40</v>
       </c>
       <c r="I34" t="str">
         <v>Expert-curated</v>
@@ -2357,7 +2394,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>max_mu</v>
+        <v>du_unbroken</v>
       </c>
       <c r="B35" t="str">
         <v>M</v>
@@ -2369,16 +2406,16 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F35">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="G35">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="H35">
-        <v>18</v>
+        <v>200</v>
       </c>
       <c r="I35" t="str">
         <v>Expert-curated</v>
@@ -2389,7 +2426,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>max_mu</v>
+        <v>du_unbroken</v>
       </c>
       <c r="B36" t="str">
         <v>F</v>
@@ -2401,16 +2438,16 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="H36">
-        <v>11</v>
+        <v>180</v>
       </c>
       <c r="I36" t="str">
         <v>Expert-curated</v>
@@ -2421,31 +2458,31 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>plank_hold</v>
+        <v>max_mu</v>
       </c>
       <c r="B37" t="str">
         <v>M</v>
       </c>
       <c r="C37" t="str">
-        <v>mm:ss</v>
+        <v>reps</v>
       </c>
       <c r="D37">
         <v>0</v>
       </c>
-      <c r="E37" t="str">
-        <v>1:00</v>
-      </c>
-      <c r="F37" t="str">
-        <v>2:00</v>
-      </c>
-      <c r="G37" t="str">
-        <v>3:00</v>
-      </c>
-      <c r="H37" t="str">
-        <v>5:00</v>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37">
+        <v>4</v>
+      </c>
+      <c r="G37">
+        <v>9</v>
+      </c>
+      <c r="H37">
+        <v>18</v>
       </c>
       <c r="I37" t="str">
-        <v>Norms + expert</v>
+        <v>Expert-curated</v>
       </c>
       <c r="J37" t="str">
         <v/>
@@ -2453,39 +2490,103 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>plank_hold</v>
+        <v>max_mu</v>
       </c>
       <c r="B38" t="str">
         <v>F</v>
       </c>
       <c r="C38" t="str">
+        <v>reps</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>5</v>
+      </c>
+      <c r="H38">
+        <v>11</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Expert-curated</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>plank_hold</v>
+      </c>
+      <c r="B39" t="str">
+        <v>M</v>
+      </c>
+      <c r="C39" t="str">
         <v>mm:ss</v>
       </c>
-      <c r="D38">
-        <v>0</v>
-      </c>
-      <c r="E38" t="str">
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39" t="str">
         <v>1:00</v>
       </c>
-      <c r="F38" t="str">
+      <c r="F39" t="str">
         <v>2:00</v>
       </c>
-      <c r="G38" t="str">
+      <c r="G39" t="str">
         <v>3:00</v>
       </c>
-      <c r="H38" t="str">
+      <c r="H39" t="str">
         <v>5:00</v>
       </c>
-      <c r="I38" t="str">
+      <c r="I39" t="str">
         <v>Norms + expert</v>
       </c>
-      <c r="J38" t="str">
+      <c r="J39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>plank_hold</v>
+      </c>
+      <c r="B40" t="str">
+        <v>F</v>
+      </c>
+      <c r="C40" t="str">
+        <v>mm:ss</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="str">
+        <v>1:00</v>
+      </c>
+      <c r="F40" t="str">
+        <v>2:00</v>
+      </c>
+      <c r="G40" t="str">
+        <v>3:00</v>
+      </c>
+      <c r="H40" t="str">
+        <v>5:00</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Norms + expert</v>
+      </c>
+      <c r="J40" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Raise CrossFit + HYROX pathway lift tiers (owner review + 2025 Games data)
CrossFit elite = Games-field level (2025 1RM squat event: 86% of men
>= 204 kg; women's podium ~160): M squat 205 / DL 240 / bench 150 /
CJ 160 / snatch 130. HYROX elite = strong end of the pro field
(McIntyre 168/238, Jacoby 127/156), not the Elite-15 median: M squat
170 / DL 210 / bench 125. Workbook Standards_Pathway rewritten +
codegen; lockstep test anchors updated. 120 tests + build green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -6104,14 +6104,14 @@
         <v>140</v>
       </c>
       <c r="H25" t="n">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="I25" t="n">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -6144,17 +6144,17 @@
         <v>68</v>
       </c>
       <c r="G26" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H26" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="I26" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -6184,20 +6184,20 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G27" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H27" t="n">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="I27" t="n">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07) (0.82x BS)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -6227,20 +6227,20 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G28" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H28" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="I28" t="n">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07) (0.82x BS)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -6276,14 +6276,14 @@
         <v>170</v>
       </c>
       <c r="H29" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="I29" t="n">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -6319,14 +6319,14 @@
         <v>114</v>
       </c>
       <c r="H30" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I30" t="n">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -6362,14 +6362,14 @@
         <v>105</v>
       </c>
       <c r="H31" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="I31" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -6405,14 +6405,14 @@
         <v>54</v>
       </c>
       <c r="H32" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I32" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -6448,14 +6448,14 @@
         <v>74</v>
       </c>
       <c r="H33" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I33" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -6491,14 +6491,14 @@
         <v>48</v>
       </c>
       <c r="H34" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I34" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -6534,14 +6534,14 @@
         <v>96</v>
       </c>
       <c r="H35" t="n">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="I35" t="n">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -6577,14 +6577,14 @@
         <v>63</v>
       </c>
       <c r="H36" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I36" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -6620,14 +6620,14 @@
         <v>85</v>
       </c>
       <c r="H37" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="I37" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -6663,14 +6663,14 @@
         <v>55</v>
       </c>
       <c r="H38" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I38" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>CrossFit athlete study (avg=good) + Games-level (2026-07)</t>
+          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -7006,20 +7006,20 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="G45" t="n">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="H45" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="I45" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -7049,20 +7049,20 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G46" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="H46" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="I46" t="n">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
@@ -7092,20 +7092,20 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="G47" t="n">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="H47" t="n">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="I47" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07) (0.82x BS)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
@@ -7135,20 +7135,20 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G48" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="H48" t="n">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I48" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07) (0.82x BS)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
@@ -7178,20 +7178,20 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="G49" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="H49" t="n">
-        <v>143</v>
+        <v>172</v>
       </c>
       <c r="I49" t="n">
-        <v>175</v>
+        <v>210</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
@@ -7221,20 +7221,20 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G50" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="I50" t="n">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
@@ -7264,20 +7264,20 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G51" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="H51" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="I51" t="n">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
@@ -7307,20 +7307,20 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G52" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="H52" t="n">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="I52" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K52" t="inlineStr"/>
@@ -7350,20 +7350,20 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G53" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H53" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I53" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
@@ -7393,20 +7393,20 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G54" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H54" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I54" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
@@ -7436,20 +7436,20 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G55" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H55" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="I55" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
@@ -7479,20 +7479,20 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G56" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="H56" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="I56" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>HYROX Elite-15 surveys, 3RM-&gt;1RM adj. (2026-07)</t>
+          <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
       <c r="K56" t="inlineStr"/>

</xml_diff>

<commit_message>
Elite = world-top-100 territory for powerlifter / crossfit / triathlete-F
Owner calibration: powerlifter elite -> IPF classic WR territory
(M 340/240/380 S/B/D; F 210/135/250); crossfit elite -> world-top-100
(M squat 230, F 165; oly lifts follow); triathlete female lifts raised
(~2xBW elite squat). Workbook + codegen + lockstep tests updated.
121 tests + build green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -6104,14 +6104,14 @@
         <v>140</v>
       </c>
       <c r="H25" t="n">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="I25" t="n">
-        <v>205</v>
+        <v>230</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -6147,14 +6147,14 @@
         <v>93</v>
       </c>
       <c r="H26" t="n">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="I26" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -6187,17 +6187,17 @@
         <v>85</v>
       </c>
       <c r="G27" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H27" t="n">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="I27" t="n">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07) (0.85x BS)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -6233,14 +6233,14 @@
         <v>79</v>
       </c>
       <c r="H28" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="I28" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07) (0.85x BS)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -6276,14 +6276,14 @@
         <v>170</v>
       </c>
       <c r="H29" t="n">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="I29" t="n">
-        <v>240</v>
+        <v>265</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -6319,14 +6319,14 @@
         <v>114</v>
       </c>
       <c r="H30" t="n">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="I30" t="n">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -6362,14 +6362,14 @@
         <v>105</v>
       </c>
       <c r="H31" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="I31" t="n">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -6405,14 +6405,14 @@
         <v>54</v>
       </c>
       <c r="H32" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="I32" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -6448,14 +6448,14 @@
         <v>74</v>
       </c>
       <c r="H33" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I33" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -6491,14 +6491,14 @@
         <v>48</v>
       </c>
       <c r="H34" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="I34" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -6534,14 +6534,14 @@
         <v>96</v>
       </c>
       <c r="H35" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="I35" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -6577,14 +6577,14 @@
         <v>63</v>
       </c>
       <c r="H36" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="I36" t="n">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -6620,14 +6620,14 @@
         <v>85</v>
       </c>
       <c r="H37" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="I37" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -6663,14 +6663,14 @@
         <v>55</v>
       </c>
       <c r="H38" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I38" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + 2025 Games-field elite (2026-07)</t>
+          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -7565,16 +7565,16 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G58" t="n">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="H58" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="I58" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -7651,16 +7651,16 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="G60" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H60" t="n">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="I60" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -7737,16 +7737,16 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="G62" t="n">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H62" t="n">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="I62" t="n">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -7823,16 +7823,16 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G64" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="H64" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="I64" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -7909,16 +7909,16 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G66" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H66" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="I66" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -7995,16 +7995,16 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G68" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="H68" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I68" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
@@ -8140,20 +8140,20 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="G71" t="n">
-        <v>160</v>
+        <v>225</v>
       </c>
       <c r="H71" t="n">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="I71" t="n">
-        <v>240</v>
+        <v>340</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
@@ -8183,20 +8183,20 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>73</v>
+        <v>105</v>
       </c>
       <c r="G72" t="n">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="H72" t="n">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="I72" t="n">
-        <v>145</v>
+        <v>210</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K72" t="inlineStr"/>
@@ -8226,20 +8226,20 @@
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="G73" t="n">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="H73" t="n">
-        <v>164</v>
+        <v>230</v>
       </c>
       <c r="I73" t="n">
-        <v>197</v>
+        <v>280</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07) (0.82x BS)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K73" t="inlineStr"/>
@@ -8269,20 +8269,20 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="G74" t="n">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="H74" t="n">
-        <v>98</v>
+        <v>141</v>
       </c>
       <c r="I74" t="n">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07) (0.82x BS)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K74" t="inlineStr"/>
@@ -8312,20 +8312,20 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>135</v>
+        <v>185</v>
       </c>
       <c r="G75" t="n">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="H75" t="n">
-        <v>230</v>
+        <v>310</v>
       </c>
       <c r="I75" t="n">
-        <v>275</v>
+        <v>380</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K75" t="inlineStr"/>
@@ -8355,20 +8355,20 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="G76" t="n">
-        <v>115</v>
+        <v>165</v>
       </c>
       <c r="H76" t="n">
-        <v>142</v>
+        <v>205</v>
       </c>
       <c r="I76" t="n">
-        <v>172</v>
+        <v>250</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K76" t="inlineStr"/>
@@ -8398,20 +8398,20 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>82</v>
+        <v>120</v>
       </c>
       <c r="G77" t="n">
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="H77" t="n">
-        <v>138</v>
+        <v>198</v>
       </c>
       <c r="I77" t="n">
-        <v>165</v>
+        <v>240</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K77" t="inlineStr"/>
@@ -8441,20 +8441,20 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="G78" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="H78" t="n">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="I78" t="n">
-        <v>88</v>
+        <v>135</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Tested feds only: van den Hoek 2024 + USAPL/IPF raw (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr"/>
@@ -8484,20 +8484,20 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="G79" t="n">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="H79" t="n">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="I79" t="n">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>SL press ladder (not contested)</t>
+          <t>Scaled to tested-elite pressing (not contested)</t>
         </is>
       </c>
       <c r="K79" t="inlineStr"/>
@@ -8527,20 +8527,20 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G80" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="H80" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="I80" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>SL press ladder (not contested)</t>
+          <t>Scaled to tested-elite pressing (not contested)</t>
         </is>
       </c>
       <c r="K80" t="inlineStr"/>

</xml_diff>

<commit_message>
Owner calibration round 3: CF peg, General rename, triathlete run ladder
CrossFit elite squat pegged 210 (participation skew; DL 245, bench 140 —
CrossFitters don't bench; oly scaled); "Gym-Goer" label -> "General"
(id gym_goer unchanged); triathlete gets its own run rows (elite mile
4:40 / 5K 16:20 M — a 5:00 mile is a hybrid ceiling, not an endurance
specialist's). Workbook + codegen + lockstep test updated.
121 tests + build green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6104,14 +6104,14 @@
         <v>140</v>
       </c>
       <c r="H25" t="n">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="I25" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -6147,14 +6147,14 @@
         <v>93</v>
       </c>
       <c r="H26" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="I26" t="n">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -6187,17 +6187,17 @@
         <v>85</v>
       </c>
       <c r="G27" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H27" t="n">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="I27" t="n">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07) (0.85x BS)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -6233,14 +6233,14 @@
         <v>79</v>
       </c>
       <c r="H28" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="I28" t="n">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07) (0.85x BS)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -6276,14 +6276,14 @@
         <v>170</v>
       </c>
       <c r="H29" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="I29" t="n">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -6319,14 +6319,14 @@
         <v>114</v>
       </c>
       <c r="H30" t="n">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="I30" t="n">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -6362,14 +6362,14 @@
         <v>105</v>
       </c>
       <c r="H31" t="n">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="I31" t="n">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07) (bench untrained in CF)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -6405,14 +6405,14 @@
         <v>54</v>
       </c>
       <c r="H32" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="I32" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07) (bench untrained in CF)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -6448,14 +6448,14 @@
         <v>74</v>
       </c>
       <c r="H33" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I33" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -6491,14 +6491,14 @@
         <v>48</v>
       </c>
       <c r="H34" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I34" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -6534,14 +6534,14 @@
         <v>96</v>
       </c>
       <c r="H35" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="I35" t="n">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -6577,14 +6577,14 @@
         <v>63</v>
       </c>
       <c r="H36" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="I36" t="n">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -6620,14 +6620,14 @@
         <v>85</v>
       </c>
       <c r="H37" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I37" t="n">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -6663,14 +6663,14 @@
         <v>55</v>
       </c>
       <c r="H38" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I38" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>CF study (avg=good) + world-top-100 elite (2026-07)</t>
+          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -8118,12 +8118,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>back_squat_1rm</t>
+          <t>run_1mi</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>powerlifter</t>
+          <t>triathlete</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -8133,27 +8133,35 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>mm:ss</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0</v>
-      </c>
-      <c r="F71" t="n">
-        <v>165</v>
-      </c>
-      <c r="G71" t="n">
-        <v>225</v>
-      </c>
-      <c r="H71" t="n">
-        <v>280</v>
-      </c>
-      <c r="I71" t="n">
-        <v>340</v>
+        <v>1</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>7:30</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>6:25</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>5:30</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>4:40</t>
+        </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
+          <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
@@ -8161,12 +8169,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>back_squat_1rm</t>
+          <t>run_1mi</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>powerlifter</t>
+          <t>triathlete</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -8176,27 +8184,35 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>mm:ss</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" t="n">
-        <v>105</v>
-      </c>
-      <c r="G72" t="n">
-        <v>140</v>
-      </c>
-      <c r="H72" t="n">
-        <v>172</v>
-      </c>
-      <c r="I72" t="n">
-        <v>210</v>
+        <v>1</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>7:30</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>6:25</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>5:30</t>
+        </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
+          <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
       <c r="K72" t="inlineStr"/>
@@ -8204,12 +8220,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>front_squat_1rm</t>
+          <t>run_5k</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>powerlifter</t>
+          <t>triathlete</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -8219,27 +8235,35 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>mm:ss</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" t="n">
-        <v>135</v>
-      </c>
-      <c r="G73" t="n">
-        <v>185</v>
-      </c>
-      <c r="H73" t="n">
-        <v>230</v>
-      </c>
-      <c r="I73" t="n">
-        <v>280</v>
+        <v>1</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>25:00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
+          <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
       <c r="K73" t="inlineStr"/>
@@ -8247,12 +8271,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>front_squat_1rm</t>
+          <t>run_5k</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>powerlifter</t>
+          <t>triathlete</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -8262,27 +8286,35 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>mm:ss</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" t="n">
-        <v>86</v>
-      </c>
-      <c r="G74" t="n">
-        <v>115</v>
-      </c>
-      <c r="H74" t="n">
-        <v>141</v>
-      </c>
-      <c r="I74" t="n">
-        <v>172</v>
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>29:00</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>24:30</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
+          <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
       <c r="K74" t="inlineStr"/>
@@ -8290,7 +8322,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>deadlift_1rm</t>
+          <t>back_squat_1rm</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -8312,16 +8344,16 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G75" t="n">
-        <v>250</v>
+        <v>225</v>
       </c>
       <c r="H75" t="n">
-        <v>310</v>
+        <v>280</v>
       </c>
       <c r="I75" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -8333,7 +8365,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>deadlift_1rm</t>
+          <t>back_squat_1rm</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -8355,16 +8387,16 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="G76" t="n">
-        <v>165</v>
+        <v>140</v>
       </c>
       <c r="H76" t="n">
-        <v>205</v>
+        <v>172</v>
       </c>
       <c r="I76" t="n">
-        <v>250</v>
+        <v>210</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -8376,7 +8408,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>bench_1rm</t>
+          <t>front_squat_1rm</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -8398,20 +8430,20 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="G77" t="n">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="H77" t="n">
-        <v>198</v>
+        <v>230</v>
       </c>
       <c r="I77" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K77" t="inlineStr"/>
@@ -8419,7 +8451,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>bench_1rm</t>
+          <t>front_squat_1rm</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -8441,20 +8473,20 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="G78" t="n">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="H78" t="n">
-        <v>110</v>
+        <v>141</v>
       </c>
       <c r="I78" t="n">
-        <v>135</v>
+        <v>172</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr"/>
@@ -8462,7 +8494,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>strict_press_1rm</t>
+          <t>deadlift_1rm</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -8484,20 +8516,20 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="G79" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="H79" t="n">
-        <v>110</v>
+        <v>310</v>
       </c>
       <c r="I79" t="n">
-        <v>135</v>
+        <v>380</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Scaled to tested-elite pressing (not contested)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K79" t="inlineStr"/>
@@ -8505,7 +8537,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>strict_press_1rm</t>
+          <t>deadlift_1rm</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -8527,20 +8559,20 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>37</v>
+        <v>122</v>
       </c>
       <c r="G80" t="n">
-        <v>50</v>
+        <v>165</v>
       </c>
       <c r="H80" t="n">
-        <v>62</v>
+        <v>205</v>
       </c>
       <c r="I80" t="n">
-        <v>75</v>
+        <v>250</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Scaled to tested-elite pressing (not contested)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K80" t="inlineStr"/>
@@ -8548,12 +8580,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>back_squat_1rm</t>
+          <t>bench_1rm</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>bodybuilder</t>
+          <t>powerlifter</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -8570,20 +8602,20 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="G81" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="H81" t="n">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="I81" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K81" t="inlineStr"/>
@@ -8591,12 +8623,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>back_squat_1rm</t>
+          <t>bench_1rm</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>bodybuilder</t>
+          <t>powerlifter</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -8613,20 +8645,20 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G82" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H82" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I82" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+          <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr"/>
@@ -8634,12 +8666,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>front_squat_1rm</t>
+          <t>strict_press_1rm</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>bodybuilder</t>
+          <t>powerlifter</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -8656,20 +8688,20 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="G83" t="n">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="H83" t="n">
-        <v>141</v>
+        <v>110</v>
       </c>
       <c r="I83" t="n">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07) (0.82x BS)</t>
+          <t>Scaled to tested-elite pressing (not contested)</t>
         </is>
       </c>
       <c r="K83" t="inlineStr"/>
@@ -8677,12 +8709,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>front_squat_1rm</t>
+          <t>strict_press_1rm</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>bodybuilder</t>
+          <t>powerlifter</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -8699,20 +8731,20 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="G84" t="n">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="H84" t="n">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="I84" t="n">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07) (0.82x BS)</t>
+          <t>Scaled to tested-elite pressing (not contested)</t>
         </is>
       </c>
       <c r="K84" t="inlineStr"/>
@@ -8720,7 +8752,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>deadlift_1rm</t>
+          <t>back_squat_1rm</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -8742,16 +8774,16 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="G85" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="H85" t="n">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="I85" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -8763,7 +8795,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>deadlift_1rm</t>
+          <t>back_squat_1rm</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -8785,16 +8817,16 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G86" t="n">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="H86" t="n">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="I86" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -8806,7 +8838,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>bench_1rm</t>
+          <t>front_squat_1rm</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -8828,20 +8860,20 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G87" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H87" t="n">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="I87" t="n">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K87" t="inlineStr"/>
@@ -8849,7 +8881,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>bench_1rm</t>
+          <t>front_squat_1rm</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -8871,20 +8903,20 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="G88" t="n">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="H88" t="n">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="I88" t="n">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07) (0.82x BS)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr"/>
@@ -8892,7 +8924,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>strict_press_1rm</t>
+          <t>deadlift_1rm</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -8914,16 +8946,16 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="G89" t="n">
-        <v>67</v>
+        <v>150</v>
       </c>
       <c r="H89" t="n">
-        <v>83</v>
+        <v>190</v>
       </c>
       <c r="I89" t="n">
-        <v>100</v>
+        <v>230</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -8935,45 +8967,217 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>deadlift_1rm</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>bodybuilder</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>75</v>
+      </c>
+      <c r="G90" t="n">
+        <v>100</v>
+      </c>
+      <c r="H90" t="n">
+        <v>123</v>
+      </c>
+      <c r="I90" t="n">
+        <v>150</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>bench_1rm</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>bodybuilder</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>80</v>
+      </c>
+      <c r="G91" t="n">
+        <v>107</v>
+      </c>
+      <c r="H91" t="n">
+        <v>132</v>
+      </c>
+      <c r="I91" t="n">
+        <v>160</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>bench_1rm</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>bodybuilder</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>42</v>
+      </c>
+      <c r="G92" t="n">
+        <v>56</v>
+      </c>
+      <c r="H92" t="n">
+        <v>69</v>
+      </c>
+      <c r="I92" t="n">
+        <v>85</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>strict_press_1rm</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>bodybuilder</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>50</v>
+      </c>
+      <c r="G93" t="n">
+        <v>67</v>
+      </c>
+      <c r="H93" t="n">
+        <v>83</v>
+      </c>
+      <c r="I93" t="n">
+        <v>100</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>strict_press_1rm</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>bodybuilder</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E90" t="n">
-        <v>0</v>
-      </c>
-      <c r="F90" t="n">
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="n">
         <v>30</v>
       </c>
-      <c r="G90" t="n">
+      <c r="G94" t="n">
         <v>40</v>
       </c>
-      <c r="H90" t="n">
+      <c r="H94" t="n">
         <v>50</v>
       </c>
-      <c r="I90" t="n">
+      <c r="I94" t="n">
         <v>62</v>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="J94" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Hybrid base bench elite -> 160 M / 90 F (owner: hybrid needs everything)
Workbook base + codegen + app-lockstep test updated. 121 tests + build green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -2565,16 +2565,16 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F17" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="G17" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="H17" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -2602,16 +2602,16 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F18" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="G18" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="H18" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CF deadlift = squat ceiling, ease all pass/good 5% (owner calibration)
CrossFit deadlift excellent/elite now tie squat's (CrossFitters barely
deadlift as a discipline); pass/good ~5% above squat's own. All pass/
good tiers across base + every pathway override eased 5% (lifts x0.95,
times x1.05) — excellent/elite untouched. Workbook + codegen +
lockstep test updated. 121 tests + build green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1984,12 +1984,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7:50</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>6:40</t>
+          <t>7:00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2029,12 +2029,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>9:25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2074,12 +2074,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>26:00</t>
+          <t>27:20</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>30:00</t>
+          <t>31:30</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>26:00</t>
+          <t>27:20</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8:00</t>
+          <t>8:25</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7:20</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2209,12 +2209,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2343,10 +2343,10 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="F11" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="G11" t="n">
         <v>155</v>
@@ -2380,10 +2380,10 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F12" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G12" t="n">
         <v>97</v>
@@ -2417,10 +2417,10 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F13" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G13" t="n">
         <v>127</v>
@@ -2454,10 +2454,10 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F14" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G14" t="n">
         <v>80</v>
@@ -2491,10 +2491,10 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="F15" t="n">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="G15" t="n">
         <v>180</v>
@@ -2528,10 +2528,10 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F16" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G16" t="n">
         <v>118</v>
@@ -2565,10 +2565,10 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F17" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
         <v>130</v>
@@ -2602,10 +2602,10 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F18" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G18" t="n">
         <v>73</v>
@@ -2639,10 +2639,10 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F19" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G19" t="n">
         <v>77</v>
@@ -2676,10 +2676,10 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F20" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G20" t="n">
         <v>45</v>
@@ -2713,10 +2713,10 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F21" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G21" t="n">
         <v>81</v>
@@ -2750,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F22" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G22" t="n">
         <v>50</v>
@@ -2787,10 +2787,10 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F23" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G23" t="n">
         <v>105</v>
@@ -2824,10 +2824,10 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F24" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G24" t="n">
         <v>66</v>
@@ -2861,10 +2861,10 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F25" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G25" t="n">
         <v>97</v>
@@ -2898,10 +2898,10 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F26" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G26" t="n">
         <v>63</v>
@@ -5104,10 +5104,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H3" t="n">
         <v>175</v>
@@ -5147,10 +5147,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G4" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H4" t="n">
         <v>102</v>
@@ -5190,10 +5190,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G5" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H5" t="n">
         <v>139</v>
@@ -5233,10 +5233,10 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G6" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H6" t="n">
         <v>82</v>
@@ -5276,10 +5276,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="G7" t="n">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="H7" t="n">
         <v>200</v>
@@ -5319,10 +5319,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G8" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="H8" t="n">
         <v>118</v>
@@ -5362,10 +5362,10 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G9" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H9" t="n">
         <v>135</v>
@@ -5405,10 +5405,10 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G10" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H10" t="n">
         <v>72</v>
@@ -5448,10 +5448,10 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G11" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H11" t="n">
         <v>88</v>
@@ -5491,10 +5491,10 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G12" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H12" t="n">
         <v>48</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="G13" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H13" t="n">
         <v>105</v>
@@ -5577,10 +5577,10 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G14" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H14" t="n">
         <v>58</v>
@@ -5620,10 +5620,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G15" t="n">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H15" t="n">
         <v>126</v>
@@ -5663,10 +5663,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G16" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H16" t="n">
         <v>72</v>
@@ -5706,10 +5706,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G17" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H17" t="n">
         <v>122</v>
@@ -5749,10 +5749,10 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G18" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H18" t="n">
         <v>70</v>
@@ -5793,12 +5793,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>9:25</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:50</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -5844,12 +5844,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -5895,12 +5895,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>30:00</t>
+          <t>31:30</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>25:00</t>
+          <t>26:15</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -5946,12 +5946,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>34:00</t>
+          <t>35:40</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>29:00</t>
+          <t>30:25</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -5997,12 +5997,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -6048,12 +6048,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>9:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -6098,10 +6098,10 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G25" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H25" t="n">
         <v>175</v>
@@ -6141,10 +6141,10 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G26" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H26" t="n">
         <v>120</v>
@@ -6184,10 +6184,10 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G27" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="H27" t="n">
         <v>148</v>
@@ -6227,10 +6227,10 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G28" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H28" t="n">
         <v>103</v>
@@ -6270,20 +6270,20 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="H29" t="n">
-        <v>205</v>
+        <v>175</v>
       </c>
       <c r="I29" t="n">
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
+          <t>same ceiling as squat, ~5% above pass/good (owner: CF barely deadlifts) (2026-07)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -6313,20 +6313,20 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G30" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="H30" t="n">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="I30" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
+          <t>same ceiling as squat, ~5% above pass/good (owner: CF barely deadlifts) (2026-07)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -6356,10 +6356,10 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G31" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H31" t="n">
         <v>122</v>
@@ -6399,10 +6399,10 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G32" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H32" t="n">
         <v>72</v>
@@ -6442,10 +6442,10 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G33" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H33" t="n">
         <v>100</v>
@@ -6485,10 +6485,10 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G34" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H34" t="n">
         <v>69</v>
@@ -6528,10 +6528,10 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G35" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="H35" t="n">
         <v>126</v>
@@ -6571,10 +6571,10 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G36" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H36" t="n">
         <v>87</v>
@@ -6614,10 +6614,10 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G37" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H37" t="n">
         <v>110</v>
@@ -6657,10 +6657,10 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G38" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H38" t="n">
         <v>75</v>
@@ -6701,12 +6701,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>7:00</t>
+          <t>7:20</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -6752,12 +6752,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>9:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>7:55</t>
+          <t>8:20</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -6803,12 +6803,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>27:00</t>
+          <t>28:20</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>24:40</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -6854,12 +6854,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>30:30</t>
+          <t>32:00</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>26:30</t>
+          <t>27:50</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -6905,12 +6905,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>7:50</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>7:10</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -6956,12 +6956,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>9:25</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -7006,10 +7006,10 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G45" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="H45" t="n">
         <v>140</v>
@@ -7049,10 +7049,10 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G46" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H46" t="n">
         <v>90</v>
@@ -7092,10 +7092,10 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G47" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H47" t="n">
         <v>115</v>
@@ -7135,10 +7135,10 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G48" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H48" t="n">
         <v>74</v>
@@ -7178,10 +7178,10 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H49" t="n">
         <v>172</v>
@@ -7221,10 +7221,10 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G50" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H50" t="n">
         <v>115</v>
@@ -7264,10 +7264,10 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G51" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H51" t="n">
         <v>102</v>
@@ -7307,10 +7307,10 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G52" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H52" t="n">
         <v>62</v>
@@ -7350,10 +7350,10 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G53" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H53" t="n">
         <v>66</v>
@@ -7393,10 +7393,10 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G54" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H54" t="n">
         <v>43</v>
@@ -7436,10 +7436,10 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G55" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H55" t="n">
         <v>86</v>
@@ -7479,10 +7479,10 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G56" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H56" t="n">
         <v>59</v>
@@ -7522,10 +7522,10 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G57" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H57" t="n">
         <v>118</v>
@@ -7565,10 +7565,10 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G58" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H58" t="n">
         <v>91</v>
@@ -7608,10 +7608,10 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G59" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H59" t="n">
         <v>97</v>
@@ -7651,10 +7651,10 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G60" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H60" t="n">
         <v>74</v>
@@ -7694,10 +7694,10 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="G61" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="H61" t="n">
         <v>146</v>
@@ -7737,10 +7737,10 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G62" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H62" t="n">
         <v>111</v>
@@ -7780,10 +7780,10 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G63" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H63" t="n">
         <v>85</v>
@@ -7823,10 +7823,10 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G64" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H64" t="n">
         <v>57</v>
@@ -7866,10 +7866,10 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G65" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H65" t="n">
         <v>57</v>
@@ -7909,10 +7909,10 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G66" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H66" t="n">
         <v>39</v>
@@ -7952,10 +7952,10 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G67" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H67" t="n">
         <v>73</v>
@@ -7995,10 +7995,10 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G68" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H68" t="n">
         <v>55</v>
@@ -8039,12 +8039,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>7:50</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>7:10</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -8090,12 +8090,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>9:25</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>8:35</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -8141,12 +8141,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:50</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>6:25</t>
+          <t>6:45</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -8192,12 +8192,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:50</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -8243,12 +8243,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>25:00</t>
+          <t>26:15</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:05</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -8294,12 +8294,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>29:00</t>
+          <t>30:25</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>24:30</t>
+          <t>25:45</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -8344,10 +8344,10 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="G75" t="n">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="H75" t="n">
         <v>280</v>
@@ -8387,10 +8387,10 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G76" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H76" t="n">
         <v>172</v>
@@ -8430,10 +8430,10 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="G77" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="H77" t="n">
         <v>230</v>
@@ -8473,10 +8473,10 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G78" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="H78" t="n">
         <v>141</v>
@@ -8516,10 +8516,10 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="G79" t="n">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="H79" t="n">
         <v>310</v>
@@ -8559,10 +8559,10 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="G80" t="n">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="H80" t="n">
         <v>205</v>
@@ -8602,10 +8602,10 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="G81" t="n">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="H81" t="n">
         <v>198</v>
@@ -8645,10 +8645,10 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G82" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H82" t="n">
         <v>110</v>
@@ -8688,10 +8688,10 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G83" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H83" t="n">
         <v>110</v>
@@ -8731,10 +8731,10 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G84" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H84" t="n">
         <v>62</v>
@@ -8774,10 +8774,10 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G85" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H85" t="n">
         <v>172</v>
@@ -8817,10 +8817,10 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G86" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="H86" t="n">
         <v>107</v>
@@ -8860,10 +8860,10 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G87" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="H87" t="n">
         <v>141</v>
@@ -8903,10 +8903,10 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G88" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="H88" t="n">
         <v>88</v>
@@ -8946,10 +8946,10 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="G89" t="n">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="H89" t="n">
         <v>190</v>
@@ -8989,10 +8989,10 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G90" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H90" t="n">
         <v>123</v>
@@ -9032,10 +9032,10 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G91" t="n">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="H91" t="n">
         <v>132</v>
@@ -9075,10 +9075,10 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G92" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H92" t="n">
         <v>69</v>
@@ -9118,10 +9118,10 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G93" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="H93" t="n">
         <v>83</v>
@@ -9161,10 +9161,10 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G94" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H94" t="n">
         <v>50</v>

</xml_diff>

<commit_message>
Round every pass/good to a multiple of 5 (owner calibration)
Same re-rounding as the app side: base + all 6 pathway overrides, kg
and seconds, nearest 5. CF deadlift-ties-squat rule corrected to apply
both the +5%-above factor and the global ease together. Workbook +
codegen + lockstep test updated. 121 tests + build green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
         <v>90</v>
       </c>
       <c r="F11" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G11" t="n">
         <v>155</v>
@@ -2380,10 +2380,10 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F12" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G12" t="n">
         <v>97</v>
@@ -2417,10 +2417,10 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F13" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G13" t="n">
         <v>127</v>
@@ -2454,10 +2454,10 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F14" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G14" t="n">
         <v>80</v>
@@ -2494,7 +2494,7 @@
         <v>105</v>
       </c>
       <c r="F15" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G15" t="n">
         <v>180</v>
@@ -2528,7 +2528,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F16" t="n">
         <v>90</v>
@@ -2565,7 +2565,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -2602,10 +2602,10 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F18" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G18" t="n">
         <v>73</v>
@@ -2639,10 +2639,10 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F19" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G19" t="n">
         <v>77</v>
@@ -2676,10 +2676,10 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F20" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G20" t="n">
         <v>45</v>
@@ -2713,10 +2713,10 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F21" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G21" t="n">
         <v>81</v>
@@ -2750,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F22" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G22" t="n">
         <v>50</v>
@@ -2787,10 +2787,10 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F23" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G23" t="n">
         <v>105</v>
@@ -2824,10 +2824,10 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F24" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G24" t="n">
         <v>66</v>
@@ -2861,10 +2861,10 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F25" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G25" t="n">
         <v>97</v>
@@ -2898,10 +2898,10 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F26" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G26" t="n">
         <v>63</v>
@@ -5107,7 +5107,7 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H3" t="n">
         <v>175</v>
@@ -5147,7 +5147,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
         <v>70</v>
@@ -5233,10 +5233,10 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G6" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H6" t="n">
         <v>82</v>
@@ -5276,10 +5276,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G7" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H7" t="n">
         <v>200</v>
@@ -5319,10 +5319,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G8" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H8" t="n">
         <v>118</v>
@@ -5362,7 +5362,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G9" t="n">
         <v>100</v>
@@ -5408,7 +5408,7 @@
         <v>30</v>
       </c>
       <c r="G10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H10" t="n">
         <v>72</v>
@@ -5448,7 +5448,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G11" t="n">
         <v>65</v>
@@ -5491,10 +5491,10 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H12" t="n">
         <v>48</v>
@@ -5534,7 +5534,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G13" t="n">
         <v>75</v>
@@ -5577,10 +5577,10 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G14" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H14" t="n">
         <v>58</v>
@@ -5620,10 +5620,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G15" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>126</v>
@@ -5663,10 +5663,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G16" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H16" t="n">
         <v>72</v>
@@ -5706,7 +5706,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G17" t="n">
         <v>90</v>
@@ -5749,10 +5749,10 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G18" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H18" t="n">
         <v>70</v>
@@ -6101,7 +6101,7 @@
         <v>95</v>
       </c>
       <c r="G25" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H25" t="n">
         <v>175</v>
@@ -6144,7 +6144,7 @@
         <v>65</v>
       </c>
       <c r="G26" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H26" t="n">
         <v>120</v>
@@ -6184,10 +6184,10 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G27" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H27" t="n">
         <v>148</v>
@@ -6313,10 +6313,10 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G30" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H30" t="n">
         <v>120</v>
@@ -6356,7 +6356,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G31" t="n">
         <v>100</v>
@@ -6399,10 +6399,10 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G32" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H32" t="n">
         <v>72</v>
@@ -6442,7 +6442,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G33" t="n">
         <v>70</v>
@@ -6485,10 +6485,10 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G34" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H34" t="n">
         <v>69</v>
@@ -6528,10 +6528,10 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G35" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H35" t="n">
         <v>126</v>
@@ -6571,7 +6571,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G36" t="n">
         <v>60</v>
@@ -6614,10 +6614,10 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G37" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H37" t="n">
         <v>110</v>
@@ -6657,10 +6657,10 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G38" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H38" t="n">
         <v>75</v>
@@ -7006,10 +7006,10 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G45" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H45" t="n">
         <v>140</v>
@@ -7049,10 +7049,10 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G46" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H46" t="n">
         <v>90</v>
@@ -7092,10 +7092,10 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G47" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H47" t="n">
         <v>115</v>
@@ -7135,10 +7135,10 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G48" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H48" t="n">
         <v>74</v>
@@ -7181,7 +7181,7 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H49" t="n">
         <v>172</v>
@@ -7221,10 +7221,10 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G50" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H50" t="n">
         <v>115</v>
@@ -7264,10 +7264,10 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G51" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H51" t="n">
         <v>102</v>
@@ -7310,7 +7310,7 @@
         <v>35</v>
       </c>
       <c r="G52" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H52" t="n">
         <v>62</v>
@@ -7350,7 +7350,7 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G53" t="n">
         <v>50</v>
@@ -7396,7 +7396,7 @@
         <v>25</v>
       </c>
       <c r="G54" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H54" t="n">
         <v>43</v>
@@ -7436,10 +7436,10 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G55" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H55" t="n">
         <v>86</v>
@@ -7479,7 +7479,7 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G56" t="n">
         <v>45</v>
@@ -7522,7 +7522,7 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G57" t="n">
         <v>90</v>
@@ -7565,10 +7565,10 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G58" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H58" t="n">
         <v>91</v>
@@ -7608,10 +7608,10 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G59" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H59" t="n">
         <v>97</v>
@@ -7651,10 +7651,10 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G60" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H60" t="n">
         <v>74</v>
@@ -7694,10 +7694,10 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G61" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H61" t="n">
         <v>146</v>
@@ -7737,7 +7737,7 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G62" t="n">
         <v>85</v>
@@ -7780,10 +7780,10 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G63" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H63" t="n">
         <v>85</v>
@@ -7823,10 +7823,10 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G64" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H64" t="n">
         <v>57</v>
@@ -7866,10 +7866,10 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G65" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H65" t="n">
         <v>57</v>
@@ -7909,10 +7909,10 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G66" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H66" t="n">
         <v>39</v>
@@ -7952,10 +7952,10 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G67" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H67" t="n">
         <v>73</v>
@@ -7998,7 +7998,7 @@
         <v>30</v>
       </c>
       <c r="G68" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H68" t="n">
         <v>55</v>
@@ -8344,10 +8344,10 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G75" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H75" t="n">
         <v>280</v>
@@ -8390,7 +8390,7 @@
         <v>100</v>
       </c>
       <c r="G76" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H76" t="n">
         <v>172</v>
@@ -8430,10 +8430,10 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G77" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H77" t="n">
         <v>230</v>
@@ -8473,10 +8473,10 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G78" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H78" t="n">
         <v>141</v>
@@ -8516,10 +8516,10 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G79" t="n">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H79" t="n">
         <v>310</v>
@@ -8559,10 +8559,10 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G80" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H80" t="n">
         <v>205</v>
@@ -8602,10 +8602,10 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G81" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H81" t="n">
         <v>198</v>
@@ -8645,7 +8645,7 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G82" t="n">
         <v>85</v>
@@ -8688,10 +8688,10 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G83" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H83" t="n">
         <v>110</v>
@@ -8734,7 +8734,7 @@
         <v>35</v>
       </c>
       <c r="G84" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H84" t="n">
         <v>62</v>
@@ -8777,7 +8777,7 @@
         <v>100</v>
       </c>
       <c r="G85" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H85" t="n">
         <v>172</v>
@@ -8817,10 +8817,10 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G86" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H86" t="n">
         <v>107</v>
@@ -8860,10 +8860,10 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G87" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H87" t="n">
         <v>141</v>
@@ -8906,7 +8906,7 @@
         <v>50</v>
       </c>
       <c r="G88" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H88" t="n">
         <v>88</v>
@@ -8946,10 +8946,10 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G89" t="n">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H89" t="n">
         <v>190</v>
@@ -8989,7 +8989,7 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G90" t="n">
         <v>95</v>

</xml_diff>

<commit_message>
HRS engine: six-tier standards, dual-mode with legacy operator/WOD curve
Supersedes the four-tier pass/good/excellent/elite scale for lift/hybrid
pathway standards — owner: the jumps between named tiers felt too big.
Beginner(pass)/Novice/Experienced(good)/Intermediate/Advanced/Elite, anchored
50/60/70/80/90/100. novice/intermediate/advanced are OPTIONAL/nullable on
ThresholdSet so operator/WOD standards (never given these values) keep
scoring on the original four-tier curve untouched — scoreHigherIsBetter/
scoreLowerIsBetter branch on novice's presence to pick the curve. `excellent`
stays required (still used by the legacy curve, vestigial on six-tier rows).

Workbook (Standards + Standards_Pathway sheets), codegen.mjs, and
BrowseStandards.tsx / format.ts UI all updated in lockstep; values match
tpf-app's hybrid_readiness.ts exactly on every shared benchmark.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1939,25 +1939,40 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>novice (60%)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>good (70%)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>excellent (85%)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>intermediate (80%)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>advanced (90%)</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>elite (100%)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>source_ref</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -1989,20 +2004,35 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>7:00</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>5:45</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>6:10</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>5:30</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>5:00</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>runninglevel/RunRepeat + 5-500 club anchor (2026-07)</t>
         </is>
@@ -2034,20 +2064,35 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>8:50</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>8:10</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>6:50</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>7:15</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>6:35</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>6:00</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>runninglevel/RunRepeat + 5-500 club anchor (2026-07)</t>
         </is>
@@ -2079,20 +2124,35 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>25:30</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>23:40</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>runninglevel/RunRepeat (2026-07)</t>
         </is>
@@ -2124,20 +2184,35 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>29:25</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>27:20</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>24:25</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>runninglevel/RunRepeat (2026-07)</t>
         </is>
@@ -2169,20 +2244,35 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>7:40</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>6:50</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>7:05</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>6:45</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>6:30</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Concept2 logbook percentiles, hybrid-adjusted (2026-07)</t>
         </is>
@@ -2214,20 +2304,35 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>8:45</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>7:45</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>7:35</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>7:15</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Concept2 logbook percentiles, hybrid-adjusted (2026-07)</t>
         </is>
@@ -2257,22 +2362,22 @@
           <t>1:50</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>1:40</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>1:33</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>1:25</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Expert + own-data</t>
         </is>
@@ -2302,22 +2407,22 @@
           <t>2:05</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>1:55</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>1:47</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>1:42</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Expert + own-data</t>
         </is>
@@ -2346,15 +2451,24 @@
         <v>90</v>
       </c>
       <c r="F11" t="n">
+        <v>105</v>
+      </c>
+      <c r="G11" t="n">
         <v>120</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>155</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
+        <v>145</v>
+      </c>
+      <c r="J11" t="n">
+        <v>165</v>
+      </c>
+      <c r="K11" t="n">
         <v>190</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2383,15 +2497,24 @@
         <v>55</v>
       </c>
       <c r="F12" t="n">
+        <v>65</v>
+      </c>
+      <c r="G12" t="n">
         <v>75</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>97</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="n">
+        <v>105</v>
+      </c>
+      <c r="K12" t="n">
         <v>120</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2420,15 +2543,24 @@
         <v>75</v>
       </c>
       <c r="F13" t="n">
+        <v>90</v>
+      </c>
+      <c r="G13" t="n">
         <v>100</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>127</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
+        <v>120</v>
+      </c>
+      <c r="J13" t="n">
+        <v>135</v>
+      </c>
+      <c r="K13" t="n">
         <v>155</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2457,15 +2589,24 @@
         <v>45</v>
       </c>
       <c r="F14" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" t="n">
         <v>60</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>80</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
+        <v>75</v>
+      </c>
+      <c r="J14" t="n">
+        <v>85</v>
+      </c>
+      <c r="K14" t="n">
         <v>98</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2494,15 +2635,24 @@
         <v>105</v>
       </c>
       <c r="F15" t="n">
+        <v>120</v>
+      </c>
+      <c r="G15" t="n">
         <v>140</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>180</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
+        <v>165</v>
+      </c>
+      <c r="J15" t="n">
+        <v>195</v>
+      </c>
+      <c r="K15" t="n">
         <v>225</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2531,15 +2681,24 @@
         <v>70</v>
       </c>
       <c r="F16" t="n">
+        <v>80</v>
+      </c>
+      <c r="G16" t="n">
         <v>90</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>118</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
+        <v>110</v>
+      </c>
+      <c r="J16" t="n">
+        <v>125</v>
+      </c>
+      <c r="K16" t="n">
         <v>145</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2568,15 +2727,24 @@
         <v>75</v>
       </c>
       <c r="F17" t="n">
+        <v>90</v>
+      </c>
+      <c r="G17" t="n">
         <v>100</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>130</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
+        <v>120</v>
+      </c>
+      <c r="J17" t="n">
+        <v>140</v>
+      </c>
+      <c r="K17" t="n">
         <v>160</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2605,15 +2773,24 @@
         <v>45</v>
       </c>
       <c r="F18" t="n">
+        <v>50</v>
+      </c>
+      <c r="G18" t="n">
         <v>55</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>73</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
+        <v>65</v>
+      </c>
+      <c r="J18" t="n">
+        <v>80</v>
+      </c>
+      <c r="K18" t="n">
         <v>90</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2642,15 +2819,24 @@
         <v>45</v>
       </c>
       <c r="F19" t="n">
+        <v>50</v>
+      </c>
+      <c r="G19" t="n">
         <v>60</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>77</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
+        <v>70</v>
+      </c>
+      <c r="J19" t="n">
+        <v>85</v>
+      </c>
+      <c r="K19" t="n">
         <v>95</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2679,15 +2865,24 @@
         <v>25</v>
       </c>
       <c r="F20" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" t="n">
         <v>35</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>45</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
+        <v>40</v>
+      </c>
+      <c r="J20" t="n">
+        <v>50</v>
+      </c>
+      <c r="K20" t="n">
         <v>55</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2716,15 +2911,24 @@
         <v>45</v>
       </c>
       <c r="F21" t="n">
+        <v>55</v>
+      </c>
+      <c r="G21" t="n">
         <v>65</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>81</v>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
+        <v>75</v>
+      </c>
+      <c r="J21" t="n">
+        <v>85</v>
+      </c>
+      <c r="K21" t="n">
         <v>100</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2753,15 +2957,24 @@
         <v>30</v>
       </c>
       <c r="F22" t="n">
+        <v>35</v>
+      </c>
+      <c r="G22" t="n">
         <v>40</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>50</v>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
+        <v>45</v>
+      </c>
+      <c r="J22" t="n">
+        <v>55</v>
+      </c>
+      <c r="K22" t="n">
         <v>62</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2790,15 +3003,24 @@
         <v>60</v>
       </c>
       <c r="F23" t="n">
+        <v>70</v>
+      </c>
+      <c r="G23" t="n">
         <v>80</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>105</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
+        <v>95</v>
+      </c>
+      <c r="J23" t="n">
+        <v>115</v>
+      </c>
+      <c r="K23" t="n">
         <v>130</v>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2827,15 +3049,24 @@
         <v>40</v>
       </c>
       <c r="F24" t="n">
+        <v>45</v>
+      </c>
+      <c r="G24" t="n">
         <v>50</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>66</v>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
+        <v>60</v>
+      </c>
+      <c r="J24" t="n">
+        <v>70</v>
+      </c>
+      <c r="K24" t="n">
         <v>82</v>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2864,15 +3095,24 @@
         <v>55</v>
       </c>
       <c r="F25" t="n">
+        <v>65</v>
+      </c>
+      <c r="G25" t="n">
         <v>75</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>97</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="n">
+        <v>105</v>
+      </c>
+      <c r="K25" t="n">
         <v>120</v>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2901,15 +3141,24 @@
         <v>35</v>
       </c>
       <c r="F26" t="n">
+        <v>40</v>
+      </c>
+      <c r="G26" t="n">
         <v>50</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>63</v>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
+        <v>60</v>
+      </c>
+      <c r="J26" t="n">
+        <v>70</v>
+      </c>
+      <c r="K26" t="n">
         <v>78</v>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>StrengthLevel/Kilgore/HYROX-CF cross-check — absolute kg, hybrid calib. (2026-07)</t>
         </is>
@@ -2937,16 +3186,16 @@
       <c r="E27" t="n">
         <v>200</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>230</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>260</v>
       </c>
-      <c r="H27" t="n">
+      <c r="K27" t="n">
         <v>285</v>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>Combine norms + expert</t>
         </is>
@@ -2974,16 +3223,16 @@
       <c r="E28" t="n">
         <v>160</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>185</v>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
         <v>210</v>
       </c>
-      <c r="H28" t="n">
+      <c r="K28" t="n">
         <v>220</v>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>Combine norms + expert</t>
         </is>
@@ -3011,16 +3260,16 @@
       <c r="E29" t="n">
         <v>5</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>11</v>
       </c>
-      <c r="G29" t="n">
+      <c r="H29" t="n">
         <v>18</v>
       </c>
-      <c r="H29" t="n">
+      <c r="K29" t="n">
         <v>25</v>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3048,16 +3297,16 @@
       <c r="E30" t="n">
         <v>1</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>5</v>
       </c>
-      <c r="G30" t="n">
+      <c r="H30" t="n">
         <v>10</v>
       </c>
-      <c r="H30" t="n">
+      <c r="K30" t="n">
         <v>18</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3085,16 +3334,16 @@
       <c r="E31" t="n">
         <v>3</v>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>8</v>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
         <v>15</v>
       </c>
-      <c r="H31" t="n">
+      <c r="K31" t="n">
         <v>25</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3122,16 +3371,16 @@
       <c r="E32" t="n">
         <v>1</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>4</v>
       </c>
-      <c r="G32" t="n">
+      <c r="H32" t="n">
         <v>8</v>
       </c>
-      <c r="H32" t="n">
+      <c r="K32" t="n">
         <v>15</v>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3159,16 +3408,16 @@
       <c r="E33" t="n">
         <v>8</v>
       </c>
-      <c r="F33" t="n">
+      <c r="G33" t="n">
         <v>18</v>
       </c>
-      <c r="G33" t="n">
+      <c r="H33" t="n">
         <v>30</v>
       </c>
-      <c r="H33" t="n">
+      <c r="K33" t="n">
         <v>45</v>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3196,16 +3445,16 @@
       <c r="E34" t="n">
         <v>5</v>
       </c>
-      <c r="F34" t="n">
+      <c r="G34" t="n">
         <v>12</v>
       </c>
-      <c r="G34" t="n">
+      <c r="H34" t="n">
         <v>22</v>
       </c>
-      <c r="H34" t="n">
+      <c r="K34" t="n">
         <v>35</v>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3233,16 +3482,16 @@
       <c r="E35" t="n">
         <v>20</v>
       </c>
-      <c r="F35" t="n">
+      <c r="G35" t="n">
         <v>50</v>
       </c>
-      <c r="G35" t="n">
+      <c r="H35" t="n">
         <v>100</v>
       </c>
-      <c r="H35" t="n">
+      <c r="K35" t="n">
         <v>150</v>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3270,16 +3519,16 @@
       <c r="E36" t="n">
         <v>15</v>
       </c>
-      <c r="F36" t="n">
+      <c r="G36" t="n">
         <v>45</v>
       </c>
-      <c r="G36" t="n">
+      <c r="H36" t="n">
         <v>90</v>
       </c>
-      <c r="H36" t="n">
+      <c r="K36" t="n">
         <v>130</v>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3307,16 +3556,16 @@
       <c r="E37" t="n">
         <v>1</v>
       </c>
-      <c r="F37" t="n">
+      <c r="G37" t="n">
         <v>4</v>
       </c>
-      <c r="G37" t="n">
+      <c r="H37" t="n">
         <v>9</v>
       </c>
-      <c r="H37" t="n">
+      <c r="K37" t="n">
         <v>14</v>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3344,16 +3593,16 @@
       <c r="E38" t="n">
         <v>1</v>
       </c>
-      <c r="F38" t="n">
+      <c r="G38" t="n">
         <v>2</v>
       </c>
-      <c r="G38" t="n">
+      <c r="H38" t="n">
         <v>5</v>
       </c>
-      <c r="H38" t="n">
+      <c r="K38" t="n">
         <v>8</v>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Expert-curated</t>
         </is>
@@ -3383,22 +3632,22 @@
           <t>1:30</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>2:30</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>3:00</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>5:00</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Norms + expert</t>
         </is>
@@ -3428,22 +3677,22 @@
           <t>1:30</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>2:30</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>3:00</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>5:00</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>Norms + expert</t>
         </is>
@@ -5012,7 +5261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5055,25 +5304,40 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>novice (60%)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>good (70%)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>excellent (85%)</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>excellent (85%, vestigial)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>intermediate (80%)</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>advanced (90%)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>elite (100%)</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>source_ref</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -5107,20 +5371,29 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
+        <v>120</v>
+      </c>
+      <c r="H3" t="n">
         <v>135</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>175</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
+        <v>160</v>
+      </c>
+      <c r="K3" t="n">
+        <v>190</v>
+      </c>
+      <c r="L3" t="n">
         <v>215</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5150,20 +5423,29 @@
         <v>50</v>
       </c>
       <c r="G4" t="n">
+        <v>60</v>
+      </c>
+      <c r="H4" t="n">
         <v>70</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>102</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
+        <v>90</v>
+      </c>
+      <c r="K4" t="n">
+        <v>110</v>
+      </c>
+      <c r="L4" t="n">
         <v>133</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5193,20 +5475,29 @@
         <v>80</v>
       </c>
       <c r="G5" t="n">
+        <v>90</v>
+      </c>
+      <c r="H5" t="n">
         <v>105</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>139</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
+        <v>130</v>
+      </c>
+      <c r="K5" t="n">
+        <v>150</v>
+      </c>
+      <c r="L5" t="n">
         <v>170</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5236,20 +5527,29 @@
         <v>45</v>
       </c>
       <c r="G6" t="n">
+        <v>50</v>
+      </c>
+      <c r="H6" t="n">
         <v>60</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>82</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
+        <v>75</v>
+      </c>
+      <c r="K6" t="n">
+        <v>90</v>
+      </c>
+      <c r="L6" t="n">
         <v>103</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5279,20 +5579,29 @@
         <v>120</v>
       </c>
       <c r="G7" t="n">
+        <v>135</v>
+      </c>
+      <c r="H7" t="n">
         <v>150</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>200</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
+        <v>185</v>
+      </c>
+      <c r="K7" t="n">
+        <v>215</v>
+      </c>
+      <c r="L7" t="n">
         <v>245</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5322,20 +5631,29 @@
         <v>60</v>
       </c>
       <c r="G8" t="n">
+        <v>70</v>
+      </c>
+      <c r="H8" t="n">
         <v>85</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>118</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
+        <v>105</v>
+      </c>
+      <c r="K8" t="n">
+        <v>130</v>
+      </c>
+      <c r="L8" t="n">
         <v>152</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5365,20 +5683,29 @@
         <v>75</v>
       </c>
       <c r="G9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H9" t="n">
         <v>100</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>135</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
+        <v>125</v>
+      </c>
+      <c r="K9" t="n">
+        <v>145</v>
+      </c>
+      <c r="L9" t="n">
         <v>165</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5408,20 +5735,29 @@
         <v>30</v>
       </c>
       <c r="G10" t="n">
+        <v>40</v>
+      </c>
+      <c r="H10" t="n">
         <v>50</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>72</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
+        <v>65</v>
+      </c>
+      <c r="K10" t="n">
+        <v>80</v>
+      </c>
+      <c r="L10" t="n">
         <v>96</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5451,20 +5787,29 @@
         <v>50</v>
       </c>
       <c r="G11" t="n">
+        <v>60</v>
+      </c>
+      <c r="H11" t="n">
         <v>65</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>88</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
+        <v>80</v>
+      </c>
+      <c r="K11" t="n">
+        <v>95</v>
+      </c>
+      <c r="L11" t="n">
         <v>110</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5494,20 +5839,29 @@
         <v>20</v>
       </c>
       <c r="G12" t="n">
+        <v>25</v>
+      </c>
+      <c r="H12" t="n">
         <v>30</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>48</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
+        <v>40</v>
+      </c>
+      <c r="K12" t="n">
+        <v>55</v>
+      </c>
+      <c r="L12" t="n">
         <v>63</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5537,20 +5891,29 @@
         <v>55</v>
       </c>
       <c r="G13" t="n">
+        <v>65</v>
+      </c>
+      <c r="H13" t="n">
         <v>75</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>105</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
+        <v>95</v>
+      </c>
+      <c r="K13" t="n">
+        <v>115</v>
+      </c>
+      <c r="L13" t="n">
         <v>133</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5580,20 +5943,29 @@
         <v>30</v>
       </c>
       <c r="G14" t="n">
+        <v>35</v>
+      </c>
+      <c r="H14" t="n">
         <v>40</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>58</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
+        <v>50</v>
+      </c>
+      <c r="K14" t="n">
+        <v>65</v>
+      </c>
+      <c r="L14" t="n">
         <v>74</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5623,20 +5995,29 @@
         <v>65</v>
       </c>
       <c r="G15" t="n">
+        <v>80</v>
+      </c>
+      <c r="H15" t="n">
         <v>90</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>126</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
+        <v>115</v>
+      </c>
+      <c r="K15" t="n">
+        <v>135</v>
+      </c>
+      <c r="L15" t="n">
         <v>158</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5666,20 +6047,29 @@
         <v>40</v>
       </c>
       <c r="G16" t="n">
+        <v>45</v>
+      </c>
+      <c r="H16" t="n">
         <v>50</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>72</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
+        <v>65</v>
+      </c>
+      <c r="K16" t="n">
+        <v>80</v>
+      </c>
+      <c r="L16" t="n">
         <v>90</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5709,20 +6099,29 @@
         <v>70</v>
       </c>
       <c r="G17" t="n">
+        <v>80</v>
+      </c>
+      <c r="H17" t="n">
         <v>90</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>122</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
+        <v>110</v>
+      </c>
+      <c r="K17" t="n">
+        <v>130</v>
+      </c>
+      <c r="L17" t="n">
         <v>150</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5752,20 +6151,29 @@
         <v>40</v>
       </c>
       <c r="G18" t="n">
+        <v>45</v>
+      </c>
+      <c r="H18" t="n">
         <v>50</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>70</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
+        <v>65</v>
+      </c>
+      <c r="K18" t="n">
+        <v>75</v>
+      </c>
+      <c r="L18" t="n">
         <v>88</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>StrengthLevel absolute ladders (2026-07)</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5793,30 +6201,45 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>9:25</t>
+          <t>9:00</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7:50</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
+          <t>7:30</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>6:30</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>6:50</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>6:15</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>5:45</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>runninglevel, gym-pop adjusted</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5844,30 +6267,45 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>7:40</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>7:25</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>6:50</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>runninglevel, gym-pop adjusted</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5895,30 +6333,45 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>31:30</t>
+          <t>30:00</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>26:15</t>
+          <t>27:30</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
+          <t>25:00</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>runninglevel, gym-pop adjusted</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5946,30 +6399,45 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>35:40</t>
+          <t>34:00</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>30:25</t>
+          <t>31:30</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
+          <t>29:00</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>25:00</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>26:20</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>24:10</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>runninglevel, gym-pop adjusted</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5997,30 +6465,45 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>8:20</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>8:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>7:05</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>7:15</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>7:00</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>6:45</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>C2 logbook, gym-pop adjusted</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6048,7 +6531,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>9:30</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6058,20 +6541,35 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>8:05</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>7:55</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>7:40</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>C2 logbook, gym-pop adjusted</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6101,20 +6599,29 @@
         <v>95</v>
       </c>
       <c r="G25" t="n">
+        <v>115</v>
+      </c>
+      <c r="H25" t="n">
         <v>135</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>175</v>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
+        <v>160</v>
+      </c>
+      <c r="K25" t="n">
+        <v>185</v>
+      </c>
+      <c r="L25" t="n">
         <v>210</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6144,20 +6651,29 @@
         <v>65</v>
       </c>
       <c r="G26" t="n">
+        <v>80</v>
+      </c>
+      <c r="H26" t="n">
         <v>90</v>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
         <v>120</v>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
+        <v>110</v>
+      </c>
+      <c r="K26" t="n">
+        <v>130</v>
+      </c>
+      <c r="L26" t="n">
         <v>150</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6187,20 +6703,29 @@
         <v>80</v>
       </c>
       <c r="G27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H27" t="n">
         <v>115</v>
       </c>
-      <c r="H27" t="n">
+      <c r="I27" t="n">
         <v>148</v>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
+        <v>135</v>
+      </c>
+      <c r="K27" t="n">
+        <v>160</v>
+      </c>
+      <c r="L27" t="n">
         <v>180</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6230,20 +6755,29 @@
         <v>55</v>
       </c>
       <c r="G28" t="n">
+        <v>65</v>
+      </c>
+      <c r="H28" t="n">
         <v>75</v>
       </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
         <v>103</v>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
+        <v>95</v>
+      </c>
+      <c r="K28" t="n">
+        <v>110</v>
+      </c>
+      <c r="L28" t="n">
         <v>128</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07) (0.85x BS)</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6273,20 +6807,29 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
+        <v>120</v>
+      </c>
+      <c r="H29" t="n">
         <v>140</v>
       </c>
-      <c r="H29" t="n">
+      <c r="I29" t="n">
         <v>175</v>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
+        <v>160</v>
+      </c>
+      <c r="K29" t="n">
+        <v>185</v>
+      </c>
+      <c r="L29" t="n">
         <v>210</v>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>same ceiling as squat, ~5% above pass/good (owner: CF barely deadlifts) (2026-07)</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>same ceiling as squat, ~5% above pass/novice (owner: CF barely deadlifts) (2026-07)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6316,20 +6859,29 @@
         <v>70</v>
       </c>
       <c r="G30" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="H30" t="n">
+        <v>93</v>
+      </c>
+      <c r="I30" t="n">
         <v>120</v>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
+        <v>110</v>
+      </c>
+      <c r="K30" t="n">
+        <v>130</v>
+      </c>
+      <c r="L30" t="n">
         <v>150</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>same ceiling as squat, ~5% above pass/good (owner: CF barely deadlifts) (2026-07)</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>same ceiling as squat, ~5% above pass/novice (owner: CF barely deadlifts) (2026-07)</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6359,20 +6911,29 @@
         <v>75</v>
       </c>
       <c r="G31" t="n">
+        <v>90</v>
+      </c>
+      <c r="H31" t="n">
         <v>100</v>
       </c>
-      <c r="H31" t="n">
+      <c r="I31" t="n">
         <v>122</v>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
+        <v>115</v>
+      </c>
+      <c r="K31" t="n">
+        <v>130</v>
+      </c>
+      <c r="L31" t="n">
         <v>140</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07) (bench untrained in CF)</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6402,20 +6963,29 @@
         <v>40</v>
       </c>
       <c r="G32" t="n">
+        <v>45</v>
+      </c>
+      <c r="H32" t="n">
         <v>50</v>
       </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>72</v>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
+        <v>65</v>
+      </c>
+      <c r="K32" t="n">
+        <v>80</v>
+      </c>
+      <c r="L32" t="n">
         <v>90</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07) (bench untrained in CF)</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6445,20 +7015,29 @@
         <v>50</v>
       </c>
       <c r="G33" t="n">
+        <v>60</v>
+      </c>
+      <c r="H33" t="n">
         <v>70</v>
       </c>
-      <c r="H33" t="n">
+      <c r="I33" t="n">
         <v>100</v>
       </c>
-      <c r="I33" t="n">
+      <c r="J33" t="n">
+        <v>90</v>
+      </c>
+      <c r="K33" t="n">
+        <v>110</v>
+      </c>
+      <c r="L33" t="n">
         <v>125</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6488,20 +7067,29 @@
         <v>35</v>
       </c>
       <c r="G34" t="n">
+        <v>40</v>
+      </c>
+      <c r="H34" t="n">
         <v>45</v>
       </c>
-      <c r="H34" t="n">
+      <c r="I34" t="n">
         <v>69</v>
       </c>
-      <c r="I34" t="n">
+      <c r="J34" t="n">
+        <v>60</v>
+      </c>
+      <c r="K34" t="n">
+        <v>75</v>
+      </c>
+      <c r="L34" t="n">
         <v>90</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6531,20 +7119,29 @@
         <v>65</v>
       </c>
       <c r="G35" t="n">
+        <v>80</v>
+      </c>
+      <c r="H35" t="n">
         <v>90</v>
       </c>
-      <c r="H35" t="n">
+      <c r="I35" t="n">
         <v>126</v>
       </c>
-      <c r="I35" t="n">
+      <c r="J35" t="n">
+        <v>115</v>
+      </c>
+      <c r="K35" t="n">
+        <v>135</v>
+      </c>
+      <c r="L35" t="n">
         <v>155</v>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6574,20 +7171,29 @@
         <v>45</v>
       </c>
       <c r="G36" t="n">
+        <v>50</v>
+      </c>
+      <c r="H36" t="n">
         <v>60</v>
       </c>
-      <c r="H36" t="n">
+      <c r="I36" t="n">
         <v>87</v>
       </c>
-      <c r="I36" t="n">
+      <c r="J36" t="n">
+        <v>80</v>
+      </c>
+      <c r="K36" t="n">
+        <v>95</v>
+      </c>
+      <c r="L36" t="n">
         <v>110</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6617,20 +7223,29 @@
         <v>60</v>
       </c>
       <c r="G37" t="n">
+        <v>70</v>
+      </c>
+      <c r="H37" t="n">
         <v>80</v>
       </c>
-      <c r="H37" t="n">
+      <c r="I37" t="n">
         <v>110</v>
       </c>
-      <c r="I37" t="n">
+      <c r="J37" t="n">
+        <v>100</v>
+      </c>
+      <c r="K37" t="n">
+        <v>120</v>
+      </c>
+      <c r="L37" t="n">
         <v>135</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6660,20 +7275,29 @@
         <v>40</v>
       </c>
       <c r="G38" t="n">
+        <v>45</v>
+      </c>
+      <c r="H38" t="n">
         <v>50</v>
       </c>
-      <c r="H38" t="n">
+      <c r="I38" t="n">
         <v>75</v>
       </c>
-      <c r="I38" t="n">
+      <c r="J38" t="n">
+        <v>65</v>
+      </c>
+      <c r="K38" t="n">
+        <v>80</v>
+      </c>
+      <c r="L38" t="n">
         <v>95</v>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>CF study (avg=good), owner-pegged elite (2026-07)</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6701,30 +7325,45 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>7:20</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
+          <t>7:00</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
           <t>6:00</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>6:20</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>5:45</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>5:20</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>CF study mile + btwb 5k pctiles</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6752,30 +7391,45 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>9:30</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
+          <t>7:55</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
           <t>6:55</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>7:15</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>6:45</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>6:20</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>CF study mile + btwb 5k pctiles</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6803,30 +7457,45 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>28:20</t>
+          <t>27:00</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>24:40</t>
+          <t>25:15</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>btwb CF 5k percentiles</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6854,30 +7523,45 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>32:00</t>
+          <t>30:30</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>27:50</t>
+          <t>28:30</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
+          <t>26:30</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
           <t>23:20</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>24:25</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>btwb CF 5k percentiles</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6905,7 +7589,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>7:50</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -6915,20 +7599,35 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
+          <t>7:10</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
           <t>6:40</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>6:50</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>6:35</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>6:20</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>Games-athlete 2k range</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6956,7 +7655,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>9:25</t>
+          <t>9:00</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -6966,20 +7665,35 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
           <t>7:45</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>7:55</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>7:35</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>7:20</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>Games-athlete 2k range</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7009,20 +7723,29 @@
         <v>80</v>
       </c>
       <c r="G45" t="n">
+        <v>90</v>
+      </c>
+      <c r="H45" t="n">
         <v>105</v>
       </c>
-      <c r="H45" t="n">
+      <c r="I45" t="n">
         <v>140</v>
       </c>
-      <c r="I45" t="n">
+      <c r="J45" t="n">
+        <v>130</v>
+      </c>
+      <c r="K45" t="n">
+        <v>150</v>
+      </c>
+      <c r="L45" t="n">
         <v>170</v>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7052,20 +7775,29 @@
         <v>50</v>
       </c>
       <c r="G46" t="n">
+        <v>60</v>
+      </c>
+      <c r="H46" t="n">
         <v>70</v>
       </c>
-      <c r="H46" t="n">
+      <c r="I46" t="n">
         <v>90</v>
       </c>
-      <c r="I46" t="n">
+      <c r="J46" t="n">
+        <v>85</v>
+      </c>
+      <c r="K46" t="n">
+        <v>95</v>
+      </c>
+      <c r="L46" t="n">
         <v>110</v>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7095,20 +7827,29 @@
         <v>65</v>
       </c>
       <c r="G47" t="n">
+        <v>80</v>
+      </c>
+      <c r="H47" t="n">
         <v>90</v>
       </c>
-      <c r="H47" t="n">
+      <c r="I47" t="n">
         <v>115</v>
       </c>
-      <c r="I47" t="n">
+      <c r="J47" t="n">
+        <v>105</v>
+      </c>
+      <c r="K47" t="n">
+        <v>125</v>
+      </c>
+      <c r="L47" t="n">
         <v>140</v>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7138,20 +7879,29 @@
         <v>45</v>
       </c>
       <c r="G48" t="n">
+        <v>50</v>
+      </c>
+      <c r="H48" t="n">
         <v>55</v>
       </c>
-      <c r="H48" t="n">
+      <c r="I48" t="n">
         <v>74</v>
       </c>
-      <c r="I48" t="n">
+      <c r="J48" t="n">
+        <v>70</v>
+      </c>
+      <c r="K48" t="n">
+        <v>80</v>
+      </c>
+      <c r="L48" t="n">
         <v>90</v>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7181,20 +7931,29 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
+        <v>120</v>
+      </c>
+      <c r="H49" t="n">
         <v>135</v>
       </c>
-      <c r="H49" t="n">
+      <c r="I49" t="n">
         <v>172</v>
       </c>
-      <c r="I49" t="n">
+      <c r="J49" t="n">
+        <v>160</v>
+      </c>
+      <c r="K49" t="n">
+        <v>185</v>
+      </c>
+      <c r="L49" t="n">
         <v>210</v>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7224,20 +7983,29 @@
         <v>65</v>
       </c>
       <c r="G50" t="n">
+        <v>75</v>
+      </c>
+      <c r="H50" t="n">
         <v>85</v>
       </c>
-      <c r="H50" t="n">
+      <c r="I50" t="n">
         <v>115</v>
       </c>
-      <c r="I50" t="n">
+      <c r="J50" t="n">
+        <v>105</v>
+      </c>
+      <c r="K50" t="n">
+        <v>125</v>
+      </c>
+      <c r="L50" t="n">
         <v>140</v>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7267,20 +8035,29 @@
         <v>60</v>
       </c>
       <c r="G51" t="n">
+        <v>70</v>
+      </c>
+      <c r="H51" t="n">
         <v>80</v>
       </c>
-      <c r="H51" t="n">
+      <c r="I51" t="n">
         <v>102</v>
       </c>
-      <c r="I51" t="n">
+      <c r="J51" t="n">
+        <v>95</v>
+      </c>
+      <c r="K51" t="n">
+        <v>110</v>
+      </c>
+      <c r="L51" t="n">
         <v>125</v>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="M51" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7310,20 +8087,29 @@
         <v>35</v>
       </c>
       <c r="G52" t="n">
+        <v>40</v>
+      </c>
+      <c r="H52" t="n">
         <v>50</v>
       </c>
-      <c r="H52" t="n">
+      <c r="I52" t="n">
         <v>62</v>
       </c>
-      <c r="I52" t="n">
+      <c r="J52" t="n">
+        <v>60</v>
+      </c>
+      <c r="K52" t="n">
+        <v>65</v>
+      </c>
+      <c r="L52" t="n">
         <v>75</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7353,20 +8139,29 @@
         <v>40</v>
       </c>
       <c r="G53" t="n">
+        <v>45</v>
+      </c>
+      <c r="H53" t="n">
         <v>50</v>
       </c>
-      <c r="H53" t="n">
+      <c r="I53" t="n">
         <v>66</v>
       </c>
-      <c r="I53" t="n">
+      <c r="J53" t="n">
+        <v>60</v>
+      </c>
+      <c r="K53" t="n">
+        <v>70</v>
+      </c>
+      <c r="L53" t="n">
         <v>80</v>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="M53" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7399,17 +8194,26 @@
         <v>30</v>
       </c>
       <c r="H54" t="n">
+        <v>30</v>
+      </c>
+      <c r="I54" t="n">
         <v>43</v>
       </c>
-      <c r="I54" t="n">
+      <c r="J54" t="n">
+        <v>40</v>
+      </c>
+      <c r="K54" t="n">
+        <v>45</v>
+      </c>
+      <c r="L54" t="n">
         <v>52</v>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7439,20 +8243,29 @@
         <v>50</v>
       </c>
       <c r="G55" t="n">
+        <v>60</v>
+      </c>
+      <c r="H55" t="n">
         <v>65</v>
       </c>
-      <c r="H55" t="n">
+      <c r="I55" t="n">
         <v>86</v>
       </c>
-      <c r="I55" t="n">
+      <c r="J55" t="n">
+        <v>80</v>
+      </c>
+      <c r="K55" t="n">
+        <v>90</v>
+      </c>
+      <c r="L55" t="n">
         <v>105</v>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="M55" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7482,20 +8295,29 @@
         <v>35</v>
       </c>
       <c r="G56" t="n">
+        <v>40</v>
+      </c>
+      <c r="H56" t="n">
         <v>45</v>
       </c>
-      <c r="H56" t="n">
+      <c r="I56" t="n">
         <v>59</v>
       </c>
-      <c r="I56" t="n">
+      <c r="J56" t="n">
+        <v>55</v>
+      </c>
+      <c r="K56" t="n">
+        <v>65</v>
+      </c>
+      <c r="L56" t="n">
         <v>72</v>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="M56" t="inlineStr">
         <is>
           <t>HYROX pro strong-end (McIntyre/Jacoby) + Elite-15 surveys (2026-07)</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7525,20 +8347,29 @@
         <v>70</v>
       </c>
       <c r="G57" t="n">
+        <v>80</v>
+      </c>
+      <c r="H57" t="n">
         <v>90</v>
       </c>
-      <c r="H57" t="n">
+      <c r="I57" t="n">
         <v>118</v>
       </c>
-      <c r="I57" t="n">
+      <c r="J57" t="n">
+        <v>110</v>
+      </c>
+      <c r="K57" t="n">
+        <v>125</v>
+      </c>
+      <c r="L57" t="n">
         <v>145</v>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="M57" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7568,20 +8399,29 @@
         <v>50</v>
       </c>
       <c r="G58" t="n">
+        <v>60</v>
+      </c>
+      <c r="H58" t="n">
         <v>70</v>
       </c>
-      <c r="H58" t="n">
+      <c r="I58" t="n">
         <v>91</v>
       </c>
-      <c r="I58" t="n">
+      <c r="J58" t="n">
+        <v>85</v>
+      </c>
+      <c r="K58" t="n">
+        <v>95</v>
+      </c>
+      <c r="L58" t="n">
         <v>110</v>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="M58" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7611,20 +8451,29 @@
         <v>55</v>
       </c>
       <c r="G59" t="n">
+        <v>65</v>
+      </c>
+      <c r="H59" t="n">
         <v>75</v>
       </c>
-      <c r="H59" t="n">
+      <c r="I59" t="n">
         <v>97</v>
       </c>
-      <c r="I59" t="n">
+      <c r="J59" t="n">
+        <v>90</v>
+      </c>
+      <c r="K59" t="n">
+        <v>105</v>
+      </c>
+      <c r="L59" t="n">
         <v>119</v>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="M59" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7654,20 +8503,29 @@
         <v>45</v>
       </c>
       <c r="G60" t="n">
+        <v>50</v>
+      </c>
+      <c r="H60" t="n">
         <v>55</v>
       </c>
-      <c r="H60" t="n">
+      <c r="I60" t="n">
         <v>74</v>
       </c>
-      <c r="I60" t="n">
+      <c r="J60" t="n">
+        <v>70</v>
+      </c>
+      <c r="K60" t="n">
+        <v>80</v>
+      </c>
+      <c r="L60" t="n">
         <v>90</v>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="M60" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7697,20 +8555,29 @@
         <v>85</v>
       </c>
       <c r="G61" t="n">
+        <v>100</v>
+      </c>
+      <c r="H61" t="n">
         <v>110</v>
       </c>
-      <c r="H61" t="n">
+      <c r="I61" t="n">
         <v>146</v>
       </c>
-      <c r="I61" t="n">
+      <c r="J61" t="n">
+        <v>135</v>
+      </c>
+      <c r="K61" t="n">
+        <v>155</v>
+      </c>
+      <c r="L61" t="n">
         <v>180</v>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="M61" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7740,20 +8607,29 @@
         <v>65</v>
       </c>
       <c r="G62" t="n">
+        <v>75</v>
+      </c>
+      <c r="H62" t="n">
         <v>85</v>
       </c>
-      <c r="H62" t="n">
+      <c r="I62" t="n">
         <v>111</v>
       </c>
-      <c r="I62" t="n">
+      <c r="J62" t="n">
+        <v>100</v>
+      </c>
+      <c r="K62" t="n">
+        <v>120</v>
+      </c>
+      <c r="L62" t="n">
         <v>135</v>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="M62" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7783,20 +8659,29 @@
         <v>50</v>
       </c>
       <c r="G63" t="n">
+        <v>60</v>
+      </c>
+      <c r="H63" t="n">
         <v>65</v>
       </c>
-      <c r="H63" t="n">
+      <c r="I63" t="n">
         <v>85</v>
       </c>
-      <c r="I63" t="n">
+      <c r="J63" t="n">
+        <v>80</v>
+      </c>
+      <c r="K63" t="n">
+        <v>90</v>
+      </c>
+      <c r="L63" t="n">
         <v>105</v>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="M63" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7826,20 +8711,29 @@
         <v>30</v>
       </c>
       <c r="G64" t="n">
+        <v>40</v>
+      </c>
+      <c r="H64" t="n">
         <v>45</v>
       </c>
-      <c r="H64" t="n">
+      <c r="I64" t="n">
         <v>57</v>
       </c>
-      <c r="I64" t="n">
+      <c r="J64" t="n">
+        <v>55</v>
+      </c>
+      <c r="K64" t="n">
+        <v>60</v>
+      </c>
+      <c r="L64" t="n">
         <v>70</v>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="M64" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7869,20 +8763,29 @@
         <v>35</v>
       </c>
       <c r="G65" t="n">
+        <v>40</v>
+      </c>
+      <c r="H65" t="n">
         <v>45</v>
       </c>
-      <c r="H65" t="n">
+      <c r="I65" t="n">
         <v>57</v>
       </c>
-      <c r="I65" t="n">
+      <c r="J65" t="n">
+        <v>55</v>
+      </c>
+      <c r="K65" t="n">
+        <v>60</v>
+      </c>
+      <c r="L65" t="n">
         <v>70</v>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="M65" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7915,17 +8818,26 @@
         <v>30</v>
       </c>
       <c r="H66" t="n">
+        <v>30</v>
+      </c>
+      <c r="I66" t="n">
         <v>39</v>
       </c>
-      <c r="I66" t="n">
+      <c r="J66" t="n">
+        <v>35</v>
+      </c>
+      <c r="K66" t="n">
+        <v>40</v>
+      </c>
+      <c r="L66" t="n">
         <v>48</v>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="M66" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7955,20 +8867,29 @@
         <v>45</v>
       </c>
       <c r="G67" t="n">
+        <v>50</v>
+      </c>
+      <c r="H67" t="n">
         <v>55</v>
       </c>
-      <c r="H67" t="n">
+      <c r="I67" t="n">
         <v>73</v>
       </c>
-      <c r="I67" t="n">
+      <c r="J67" t="n">
+        <v>65</v>
+      </c>
+      <c r="K67" t="n">
+        <v>80</v>
+      </c>
+      <c r="L67" t="n">
         <v>90</v>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="M67" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7998,20 +8919,29 @@
         <v>30</v>
       </c>
       <c r="G68" t="n">
+        <v>35</v>
+      </c>
+      <c r="H68" t="n">
         <v>40</v>
       </c>
-      <c r="H68" t="n">
+      <c r="I68" t="n">
         <v>55</v>
       </c>
-      <c r="I68" t="n">
+      <c r="J68" t="n">
+        <v>50</v>
+      </c>
+      <c r="K68" t="n">
+        <v>60</v>
+      </c>
+      <c r="L68" t="n">
         <v>66</v>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="M68" t="inlineStr">
         <is>
           <t>Endurance-athlete strength profile (2026-07)</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8039,7 +8969,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>7:50</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -8049,20 +8979,35 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
+          <t>7:10</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
           <t>6:40</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>6:50</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>6:35</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>6:20</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="M69" t="inlineStr">
         <is>
           <t>C2 logbook, engine-athlete tier</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8090,7 +9035,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>9:25</t>
+          <t>9:00</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -8100,20 +9045,35 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
           <t>7:35</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>7:25</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
         <is>
           <t>7:05</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="M70" t="inlineStr">
         <is>
           <t>C2 logbook, engine-athlete tier</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8141,30 +9101,45 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>7:50</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>6:45</t>
+          <t>7:00</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
+          <t>6:25</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
           <t>5:30</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>5:50</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>5:15</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
         <is>
           <t>4:40</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="M71" t="inlineStr">
         <is>
           <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8192,30 +9167,45 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>7:50</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
+          <t>7:30</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
           <t>6:25</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>6:45</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>6:05</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>5:30</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="M72" t="inlineStr">
         <is>
           <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8243,30 +9233,45 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>26:15</t>
+          <t>25:00</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>22:05</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
           <t>18:20</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>16:20</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="M73" t="inlineStr">
         <is>
           <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8294,30 +9299,45 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>30:25</t>
+          <t>29:00</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>25:45</t>
+          <t>26:45</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
+          <t>24:30</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>19:20</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="M74" t="inlineStr">
         <is>
           <t>Elite AG/pro standalone run ability</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8347,20 +9367,29 @@
         <v>155</v>
       </c>
       <c r="G75" t="n">
+        <v>185</v>
+      </c>
+      <c r="H75" t="n">
         <v>215</v>
       </c>
-      <c r="H75" t="n">
+      <c r="I75" t="n">
         <v>280</v>
       </c>
-      <c r="I75" t="n">
+      <c r="J75" t="n">
+        <v>260</v>
+      </c>
+      <c r="K75" t="n">
+        <v>300</v>
+      </c>
+      <c r="L75" t="n">
         <v>340</v>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="M75" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8390,20 +9419,29 @@
         <v>100</v>
       </c>
       <c r="G76" t="n">
+        <v>120</v>
+      </c>
+      <c r="H76" t="n">
         <v>135</v>
       </c>
-      <c r="H76" t="n">
+      <c r="I76" t="n">
         <v>172</v>
       </c>
-      <c r="I76" t="n">
+      <c r="J76" t="n">
+        <v>160</v>
+      </c>
+      <c r="K76" t="n">
+        <v>185</v>
+      </c>
+      <c r="L76" t="n">
         <v>210</v>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="M76" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8433,20 +9471,29 @@
         <v>130</v>
       </c>
       <c r="G77" t="n">
+        <v>150</v>
+      </c>
+      <c r="H77" t="n">
         <v>175</v>
       </c>
-      <c r="H77" t="n">
+      <c r="I77" t="n">
         <v>230</v>
       </c>
-      <c r="I77" t="n">
+      <c r="J77" t="n">
+        <v>210</v>
+      </c>
+      <c r="K77" t="n">
+        <v>245</v>
+      </c>
+      <c r="L77" t="n">
         <v>280</v>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="M77" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8476,20 +9523,29 @@
         <v>80</v>
       </c>
       <c r="G78" t="n">
+        <v>95</v>
+      </c>
+      <c r="H78" t="n">
         <v>110</v>
       </c>
-      <c r="H78" t="n">
+      <c r="I78" t="n">
         <v>141</v>
       </c>
-      <c r="I78" t="n">
+      <c r="J78" t="n">
+        <v>130</v>
+      </c>
+      <c r="K78" t="n">
+        <v>150</v>
+      </c>
+      <c r="L78" t="n">
         <v>172</v>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="M78" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8519,20 +9575,29 @@
         <v>175</v>
       </c>
       <c r="G79" t="n">
+        <v>210</v>
+      </c>
+      <c r="H79" t="n">
         <v>240</v>
       </c>
-      <c r="H79" t="n">
+      <c r="I79" t="n">
         <v>310</v>
       </c>
-      <c r="I79" t="n">
+      <c r="J79" t="n">
+        <v>285</v>
+      </c>
+      <c r="K79" t="n">
+        <v>335</v>
+      </c>
+      <c r="L79" t="n">
         <v>380</v>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="M79" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8562,20 +9627,29 @@
         <v>115</v>
       </c>
       <c r="G80" t="n">
+        <v>135</v>
+      </c>
+      <c r="H80" t="n">
         <v>155</v>
       </c>
-      <c r="H80" t="n">
+      <c r="I80" t="n">
         <v>205</v>
       </c>
-      <c r="I80" t="n">
+      <c r="J80" t="n">
+        <v>190</v>
+      </c>
+      <c r="K80" t="n">
+        <v>220</v>
+      </c>
+      <c r="L80" t="n">
         <v>250</v>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="M80" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8605,20 +9679,29 @@
         <v>115</v>
       </c>
       <c r="G81" t="n">
+        <v>130</v>
+      </c>
+      <c r="H81" t="n">
         <v>150</v>
       </c>
-      <c r="H81" t="n">
+      <c r="I81" t="n">
         <v>198</v>
       </c>
-      <c r="I81" t="n">
+      <c r="J81" t="n">
+        <v>180</v>
+      </c>
+      <c r="K81" t="n">
+        <v>210</v>
+      </c>
+      <c r="L81" t="n">
         <v>240</v>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="M81" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8648,20 +9731,29 @@
         <v>65</v>
       </c>
       <c r="G82" t="n">
+        <v>75</v>
+      </c>
+      <c r="H82" t="n">
         <v>85</v>
       </c>
-      <c r="H82" t="n">
+      <c r="I82" t="n">
         <v>110</v>
       </c>
-      <c r="I82" t="n">
+      <c r="J82" t="n">
+        <v>100</v>
+      </c>
+      <c r="K82" t="n">
+        <v>120</v>
+      </c>
+      <c r="L82" t="n">
         <v>135</v>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="M82" t="inlineStr">
         <is>
           <t>Tested world-class: IPF classic WRs + USAPL nats (2026-07)</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8691,20 +9783,29 @@
         <v>60</v>
       </c>
       <c r="G83" t="n">
+        <v>70</v>
+      </c>
+      <c r="H83" t="n">
         <v>85</v>
       </c>
-      <c r="H83" t="n">
+      <c r="I83" t="n">
         <v>110</v>
       </c>
-      <c r="I83" t="n">
+      <c r="J83" t="n">
+        <v>100</v>
+      </c>
+      <c r="K83" t="n">
+        <v>120</v>
+      </c>
+      <c r="L83" t="n">
         <v>135</v>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="M83" t="inlineStr">
         <is>
           <t>Scaled to tested-elite pressing (not contested)</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8734,20 +9835,29 @@
         <v>35</v>
       </c>
       <c r="G84" t="n">
+        <v>40</v>
+      </c>
+      <c r="H84" t="n">
         <v>50</v>
       </c>
-      <c r="H84" t="n">
+      <c r="I84" t="n">
         <v>62</v>
       </c>
-      <c r="I84" t="n">
+      <c r="J84" t="n">
+        <v>60</v>
+      </c>
+      <c r="K84" t="n">
+        <v>65</v>
+      </c>
+      <c r="L84" t="n">
         <v>75</v>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="M84" t="inlineStr">
         <is>
           <t>Scaled to tested-elite pressing (not contested)</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8777,20 +9887,29 @@
         <v>100</v>
       </c>
       <c r="G85" t="n">
+        <v>120</v>
+      </c>
+      <c r="H85" t="n">
         <v>135</v>
       </c>
-      <c r="H85" t="n">
+      <c r="I85" t="n">
         <v>172</v>
       </c>
-      <c r="I85" t="n">
+      <c r="J85" t="n">
+        <v>160</v>
+      </c>
+      <c r="K85" t="n">
+        <v>185</v>
+      </c>
+      <c r="L85" t="n">
         <v>210</v>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="M85" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -8820,20 +9939,29 @@
         <v>60</v>
       </c>
       <c r="G86" t="n">
+        <v>70</v>
+      </c>
+      <c r="H86" t="n">
         <v>85</v>
       </c>
-      <c r="H86" t="n">
+      <c r="I86" t="n">
         <v>107</v>
       </c>
-      <c r="I86" t="n">
+      <c r="J86" t="n">
+        <v>100</v>
+      </c>
+      <c r="K86" t="n">
+        <v>115</v>
+      </c>
+      <c r="L86" t="n">
         <v>130</v>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="M86" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8863,20 +9991,29 @@
         <v>80</v>
       </c>
       <c r="G87" t="n">
+        <v>95</v>
+      </c>
+      <c r="H87" t="n">
         <v>110</v>
       </c>
-      <c r="H87" t="n">
+      <c r="I87" t="n">
         <v>141</v>
       </c>
-      <c r="I87" t="n">
+      <c r="J87" t="n">
+        <v>130</v>
+      </c>
+      <c r="K87" t="n">
+        <v>150</v>
+      </c>
+      <c r="L87" t="n">
         <v>172</v>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="M87" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8906,20 +10043,29 @@
         <v>50</v>
       </c>
       <c r="G88" t="n">
+        <v>60</v>
+      </c>
+      <c r="H88" t="n">
         <v>65</v>
       </c>
-      <c r="H88" t="n">
+      <c r="I88" t="n">
         <v>88</v>
       </c>
-      <c r="I88" t="n">
+      <c r="J88" t="n">
+        <v>80</v>
+      </c>
+      <c r="K88" t="n">
+        <v>95</v>
+      </c>
+      <c r="L88" t="n">
         <v>107</v>
       </c>
-      <c r="J88" t="inlineStr">
+      <c r="M88" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07) (0.82x BS)</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8949,20 +10095,29 @@
         <v>110</v>
       </c>
       <c r="G89" t="n">
+        <v>125</v>
+      </c>
+      <c r="H89" t="n">
         <v>140</v>
       </c>
-      <c r="H89" t="n">
+      <c r="I89" t="n">
         <v>190</v>
       </c>
-      <c r="I89" t="n">
+      <c r="J89" t="n">
+        <v>175</v>
+      </c>
+      <c r="K89" t="n">
+        <v>205</v>
+      </c>
+      <c r="L89" t="n">
         <v>230</v>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="M89" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8992,20 +10147,29 @@
         <v>70</v>
       </c>
       <c r="G90" t="n">
+        <v>80</v>
+      </c>
+      <c r="H90" t="n">
         <v>95</v>
       </c>
-      <c r="H90" t="n">
+      <c r="I90" t="n">
         <v>123</v>
       </c>
-      <c r="I90" t="n">
+      <c r="J90" t="n">
+        <v>115</v>
+      </c>
+      <c r="K90" t="n">
+        <v>130</v>
+      </c>
+      <c r="L90" t="n">
         <v>150</v>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="M90" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9035,20 +10199,29 @@
         <v>76</v>
       </c>
       <c r="G91" t="n">
+        <v>90</v>
+      </c>
+      <c r="H91" t="n">
         <v>102</v>
       </c>
-      <c r="H91" t="n">
+      <c r="I91" t="n">
         <v>132</v>
       </c>
-      <c r="I91" t="n">
+      <c r="J91" t="n">
+        <v>120</v>
+      </c>
+      <c r="K91" t="n">
+        <v>140</v>
+      </c>
+      <c r="L91" t="n">
         <v>160</v>
       </c>
-      <c r="J91" t="inlineStr">
+      <c r="M91" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -9078,20 +10251,29 @@
         <v>40</v>
       </c>
       <c r="G92" t="n">
+        <v>45</v>
+      </c>
+      <c r="H92" t="n">
         <v>53</v>
       </c>
-      <c r="H92" t="n">
+      <c r="I92" t="n">
         <v>69</v>
       </c>
-      <c r="I92" t="n">
+      <c r="J92" t="n">
+        <v>65</v>
+      </c>
+      <c r="K92" t="n">
+        <v>75</v>
+      </c>
+      <c r="L92" t="n">
         <v>85</v>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="M92" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9121,20 +10303,29 @@
         <v>48</v>
       </c>
       <c r="G93" t="n">
+        <v>55</v>
+      </c>
+      <c r="H93" t="n">
         <v>64</v>
       </c>
-      <c r="H93" t="n">
+      <c r="I93" t="n">
         <v>83</v>
       </c>
-      <c r="I93" t="n">
+      <c r="J93" t="n">
+        <v>75</v>
+      </c>
+      <c r="K93" t="n">
+        <v>90</v>
+      </c>
+      <c r="L93" t="n">
         <v>100</v>
       </c>
-      <c r="J93" t="inlineStr">
+      <c r="M93" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9164,20 +10355,29 @@
         <v>29</v>
       </c>
       <c r="G94" t="n">
+        <v>35</v>
+      </c>
+      <c r="H94" t="n">
         <v>38</v>
       </c>
-      <c r="H94" t="n">
+      <c r="I94" t="n">
         <v>50</v>
       </c>
-      <c r="I94" t="n">
+      <c r="J94" t="n">
+        <v>45</v>
+      </c>
+      <c r="K94" t="n">
+        <v>55</v>
+      </c>
+      <c r="L94" t="n">
         <v>62</v>
       </c>
-      <c r="J94" t="inlineStr">
+      <c r="M94" t="inlineStr">
         <is>
           <t>Natural BB standards (M&amp;S natural ladder, Henselmans) (2026-07)</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
HRS: shift Beginner down 10%, Novice down 5%; fix strict_press lockstep bug
Owner: both tiers read too demanding. Applied to base + all pathway
overrides, rounded to nearest 5/5s; Good/Intermediate/Advanced/Elite
untouched. Also fixes a pre-existing lockstep bug found while verifying
the shift: hyrox/triathlete F strict_press novice was 30 here (tying
`good`=30) but 27 in tpf-app — corrected to 27 before shifting.

Strengthened the "override tier set ordered" test to strict pairwise
comparisons (was a sort-equality check, which can't catch exact ties)
and to actually examine novice/intermediate/advanced — this test would
have caught the bug above had it existed at the time.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1999,12 +1999,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9:25</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>8:50</t>
+          <t>9:15</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>27:20</t>
+          <t>30:05</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>25:30</t>
+          <t>26:45</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>31:30</t>
+          <t>34:40</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>29:25</t>
+          <t>30:55</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2239,12 +2239,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>9:15</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>8:25</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>8:00</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2299,12 +2299,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>9:40</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>9:10</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2448,10 +2448,10 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G11" t="n">
         <v>120</v>
@@ -2494,10 +2494,10 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G12" t="n">
         <v>75</v>
@@ -2540,10 +2540,10 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F13" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G13" t="n">
         <v>100</v>
@@ -2586,7 +2586,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F14" t="n">
         <v>50</v>
@@ -2632,10 +2632,10 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="F15" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G15" t="n">
         <v>140</v>
@@ -2678,10 +2678,10 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F16" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G16" t="n">
         <v>90</v>
@@ -2724,10 +2724,10 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F17" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G17" t="n">
         <v>100</v>
@@ -2770,7 +2770,7 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F18" t="n">
         <v>50</v>
@@ -2816,7 +2816,7 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F19" t="n">
         <v>50</v>
@@ -2862,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F20" t="n">
         <v>30</v>
@@ -2908,10 +2908,10 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F21" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G21" t="n">
         <v>65</v>
@@ -2954,7 +2954,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F22" t="n">
         <v>35</v>
@@ -3000,10 +3000,10 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F23" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G23" t="n">
         <v>80</v>
@@ -3046,7 +3046,7 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F24" t="n">
         <v>45</v>
@@ -3092,10 +3092,10 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F25" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G25" t="n">
         <v>75</v>
@@ -3138,7 +3138,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F26" t="n">
         <v>40</v>
@@ -5368,10 +5368,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G3" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H3" t="n">
         <v>135</v>
@@ -5420,10 +5420,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G4" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -5472,10 +5472,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H5" t="n">
         <v>105</v>
@@ -5524,7 +5524,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G6" t="n">
         <v>50</v>
@@ -5576,10 +5576,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="G7" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="H7" t="n">
         <v>150</v>
@@ -5628,10 +5628,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G8" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H8" t="n">
         <v>85</v>
@@ -5680,10 +5680,10 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G9" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H9" t="n">
         <v>100</v>
@@ -5732,7 +5732,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G10" t="n">
         <v>40</v>
@@ -5784,10 +5784,10 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G11" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H11" t="n">
         <v>65</v>
@@ -5888,10 +5888,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G13" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H13" t="n">
         <v>75</v>
@@ -5940,7 +5940,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G14" t="n">
         <v>35</v>
@@ -5992,10 +5992,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G15" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H15" t="n">
         <v>90</v>
@@ -6044,7 +6044,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G16" t="n">
         <v>45</v>
@@ -6096,10 +6096,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G17" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H17" t="n">
         <v>90</v>
@@ -6148,7 +6148,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G18" t="n">
         <v>45</v>
@@ -6201,12 +6201,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>9:55</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -6267,12 +6267,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -6333,12 +6333,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>30:00</t>
+          <t>33:00</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>27:30</t>
+          <t>28:50</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -6399,12 +6399,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>34:00</t>
+          <t>37:25</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>31:30</t>
+          <t>33:05</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -6465,12 +6465,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8:00</t>
+          <t>8:25</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -6531,12 +6531,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>9:30</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -6596,10 +6596,10 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="G25" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="H25" t="n">
         <v>135</v>
@@ -6648,10 +6648,10 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G26" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H26" t="n">
         <v>90</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G27" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H27" t="n">
         <v>115</v>
@@ -6752,10 +6752,10 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G28" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H28" t="n">
         <v>75</v>
@@ -6804,10 +6804,10 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G29" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H29" t="n">
         <v>140</v>
@@ -6856,10 +6856,10 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G30" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H30" t="n">
         <v>93</v>
@@ -6908,10 +6908,10 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G31" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H31" t="n">
         <v>100</v>
@@ -6960,7 +6960,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G32" t="n">
         <v>45</v>
@@ -7012,10 +7012,10 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G33" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H33" t="n">
         <v>70</v>
@@ -7064,7 +7064,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G34" t="n">
         <v>40</v>
@@ -7116,10 +7116,10 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G35" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H35" t="n">
         <v>90</v>
@@ -7168,7 +7168,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G36" t="n">
         <v>50</v>
@@ -7220,10 +7220,10 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G37" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H37" t="n">
         <v>80</v>
@@ -7272,7 +7272,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G38" t="n">
         <v>45</v>
@@ -7325,12 +7325,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -7391,12 +7391,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>9:30</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -7457,12 +7457,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>27:00</t>
+          <t>29:40</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>25:15</t>
+          <t>26:30</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -7523,12 +7523,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>30:30</t>
+          <t>33:35</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>28:30</t>
+          <t>29:55</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -7589,12 +7589,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
+          <t>8:35</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>7:50</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>7:30</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -7655,12 +7655,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>9:55</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -7720,10 +7720,10 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G45" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H45" t="n">
         <v>105</v>
@@ -7772,10 +7772,10 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G46" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H46" t="n">
         <v>70</v>
@@ -7824,10 +7824,10 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G47" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H47" t="n">
         <v>90</v>
@@ -7876,7 +7876,7 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G48" t="n">
         <v>50</v>
@@ -7928,10 +7928,10 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G49" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H49" t="n">
         <v>135</v>
@@ -7980,10 +7980,10 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G50" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H50" t="n">
         <v>85</v>
@@ -8032,10 +8032,10 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G51" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H51" t="n">
         <v>80</v>
@@ -8084,7 +8084,7 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G52" t="n">
         <v>40</v>
@@ -8136,7 +8136,7 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G53" t="n">
         <v>45</v>
@@ -8188,10 +8188,10 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
+        <v>20</v>
+      </c>
+      <c r="G54" t="n">
         <v>25</v>
-      </c>
-      <c r="G54" t="n">
-        <v>30</v>
       </c>
       <c r="H54" t="n">
         <v>30</v>
@@ -8240,10 +8240,10 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G55" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H55" t="n">
         <v>65</v>
@@ -8292,7 +8292,7 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G56" t="n">
         <v>40</v>
@@ -8344,10 +8344,10 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G57" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H57" t="n">
         <v>90</v>
@@ -8396,10 +8396,10 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G58" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H58" t="n">
         <v>70</v>
@@ -8448,10 +8448,10 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G59" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H59" t="n">
         <v>75</v>
@@ -8500,7 +8500,7 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G60" t="n">
         <v>50</v>
@@ -8552,10 +8552,10 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G61" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H61" t="n">
         <v>110</v>
@@ -8604,10 +8604,10 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G62" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H62" t="n">
         <v>85</v>
@@ -8656,10 +8656,10 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G63" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H63" t="n">
         <v>65</v>
@@ -8708,7 +8708,7 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G64" t="n">
         <v>40</v>
@@ -8760,7 +8760,7 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G65" t="n">
         <v>40</v>
@@ -8812,10 +8812,10 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
+        <v>20</v>
+      </c>
+      <c r="G66" t="n">
         <v>25</v>
-      </c>
-      <c r="G66" t="n">
-        <v>30</v>
       </c>
       <c r="H66" t="n">
         <v>30</v>
@@ -8864,7 +8864,7 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G67" t="n">
         <v>50</v>
@@ -8916,7 +8916,7 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G68" t="n">
         <v>35</v>
@@ -8969,12 +8969,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
+          <t>8:35</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
           <t>7:50</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>7:30</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -9035,12 +9035,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
+          <t>9:55</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
           <t>9:00</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>8:35</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -9101,12 +9101,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>7:00</t>
+          <t>7:20</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -9167,12 +9167,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>9:30</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>8:30</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -9233,12 +9233,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>25:00</t>
+          <t>27:30</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>24:10</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -9299,12 +9299,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>29:00</t>
+          <t>31:55</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>26:45</t>
+          <t>28:05</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -9364,10 +9364,10 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="G75" t="n">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="H75" t="n">
         <v>215</v>
@@ -9416,10 +9416,10 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G76" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H76" t="n">
         <v>135</v>
@@ -9468,10 +9468,10 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="G77" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="H77" t="n">
         <v>175</v>
@@ -9520,10 +9520,10 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G78" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H78" t="n">
         <v>110</v>
@@ -9572,10 +9572,10 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="G79" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="H79" t="n">
         <v>240</v>
@@ -9624,10 +9624,10 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="G80" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="H80" t="n">
         <v>155</v>
@@ -9676,10 +9676,10 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="G81" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="H81" t="n">
         <v>150</v>
@@ -9728,10 +9728,10 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G82" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H82" t="n">
         <v>85</v>
@@ -9780,10 +9780,10 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G83" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H83" t="n">
         <v>85</v>
@@ -9832,7 +9832,7 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G84" t="n">
         <v>40</v>
@@ -9884,10 +9884,10 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G85" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H85" t="n">
         <v>135</v>
@@ -9936,10 +9936,10 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G86" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H86" t="n">
         <v>85</v>
@@ -9988,10 +9988,10 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G87" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H87" t="n">
         <v>110</v>
@@ -10040,10 +10040,10 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G88" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H88" t="n">
         <v>65</v>
@@ -10092,10 +10092,10 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G89" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H89" t="n">
         <v>140</v>
@@ -10144,10 +10144,10 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G90" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H90" t="n">
         <v>95</v>
@@ -10196,10 +10196,10 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G91" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H91" t="n">
         <v>102</v>
@@ -10248,7 +10248,7 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G92" t="n">
         <v>45</v>
@@ -10300,10 +10300,10 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G93" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H93" t="n">
         <v>64</v>
@@ -10352,7 +10352,7 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G94" t="n">
         <v>35</v>

</xml_diff>

<commit_message>
HRS: widen powerlifter scale — Beginner should read as beginner
Owner: Beginner still read as strength-athlete-experienced (140 kg squat),
not a true "just started powerlifting" number. Elite unchanged (already
researched world-class); every other tier re-derived from a hand-designed
Beginner->Elite back-squat ladder with each other lift scaled by its own
existing elite:squat ratio. Vestigial `excellent` recomputed as the
good/intermediate midpoint so the browse-standards table doesn't show an
orphaned out-of-order number for this pathway.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -9364,22 +9364,22 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="G75" t="n">
-        <v>175</v>
+        <v>90</v>
       </c>
       <c r="H75" t="n">
-        <v>215</v>
+        <v>130</v>
       </c>
       <c r="I75" t="n">
-        <v>280</v>
+        <v>155</v>
       </c>
       <c r="J75" t="n">
-        <v>260</v>
+        <v>180</v>
       </c>
       <c r="K75" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="L75" t="n">
         <v>340</v>
@@ -9416,22 +9416,22 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="G76" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="H76" t="n">
-        <v>135</v>
+        <v>85</v>
       </c>
       <c r="I76" t="n">
-        <v>172</v>
+        <v>100</v>
       </c>
       <c r="J76" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="K76" t="n">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="L76" t="n">
         <v>210</v>
@@ -9468,22 +9468,22 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="G77" t="n">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="H77" t="n">
-        <v>175</v>
+        <v>105</v>
       </c>
       <c r="I77" t="n">
-        <v>230</v>
+        <v>130</v>
       </c>
       <c r="J77" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="K77" t="n">
-        <v>245</v>
+        <v>205</v>
       </c>
       <c r="L77" t="n">
         <v>280</v>
@@ -9520,22 +9520,22 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
+        <v>35</v>
+      </c>
+      <c r="G78" t="n">
+        <v>50</v>
+      </c>
+      <c r="H78" t="n">
         <v>70</v>
       </c>
-      <c r="G78" t="n">
-        <v>90</v>
-      </c>
-      <c r="H78" t="n">
-        <v>110</v>
-      </c>
       <c r="I78" t="n">
-        <v>141</v>
+        <v>85</v>
       </c>
       <c r="J78" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="K78" t="n">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="L78" t="n">
         <v>172</v>
@@ -9572,22 +9572,22 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>160</v>
+        <v>65</v>
       </c>
       <c r="G79" t="n">
+        <v>100</v>
+      </c>
+      <c r="H79" t="n">
+        <v>145</v>
+      </c>
+      <c r="I79" t="n">
+        <v>170</v>
+      </c>
+      <c r="J79" t="n">
         <v>200</v>
       </c>
-      <c r="H79" t="n">
-        <v>240</v>
-      </c>
-      <c r="I79" t="n">
-        <v>310</v>
-      </c>
-      <c r="J79" t="n">
-        <v>285</v>
-      </c>
       <c r="K79" t="n">
-        <v>335</v>
+        <v>280</v>
       </c>
       <c r="L79" t="n">
         <v>380</v>
@@ -9624,22 +9624,22 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="G80" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="H80" t="n">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="I80" t="n">
-        <v>205</v>
+        <v>120</v>
       </c>
       <c r="J80" t="n">
-        <v>190</v>
+        <v>145</v>
       </c>
       <c r="K80" t="n">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="L80" t="n">
         <v>250</v>
@@ -9676,22 +9676,22 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="G81" t="n">
+        <v>65</v>
+      </c>
+      <c r="H81" t="n">
+        <v>90</v>
+      </c>
+      <c r="I81" t="n">
+        <v>110</v>
+      </c>
+      <c r="J81" t="n">
         <v>125</v>
       </c>
-      <c r="H81" t="n">
-        <v>150</v>
-      </c>
-      <c r="I81" t="n">
-        <v>198</v>
-      </c>
-      <c r="J81" t="n">
-        <v>180</v>
-      </c>
       <c r="K81" t="n">
-        <v>210</v>
+        <v>175</v>
       </c>
       <c r="L81" t="n">
         <v>240</v>
@@ -9728,22 +9728,22 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="G82" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H82" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="I82" t="n">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="J82" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="K82" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="L82" t="n">
         <v>135</v>
@@ -9780,22 +9780,22 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G83" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="H83" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="I83" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="J83" t="n">
+        <v>70</v>
+      </c>
+      <c r="K83" t="n">
         <v>100</v>
-      </c>
-      <c r="K83" t="n">
-        <v>120</v>
       </c>
       <c r="L83" t="n">
         <v>135</v>
@@ -9832,22 +9832,22 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
+        <v>15</v>
+      </c>
+      <c r="G84" t="n">
+        <v>20</v>
+      </c>
+      <c r="H84" t="n">
         <v>30</v>
       </c>
-      <c r="G84" t="n">
+      <c r="I84" t="n">
         <v>40</v>
       </c>
-      <c r="H84" t="n">
-        <v>50</v>
-      </c>
-      <c r="I84" t="n">
-        <v>62</v>
-      </c>
       <c r="J84" t="n">
+        <v>45</v>
+      </c>
+      <c r="K84" t="n">
         <v>60</v>
-      </c>
-      <c r="K84" t="n">
-        <v>65</v>
       </c>
       <c r="L84" t="n">
         <v>75</v>

</xml_diff>

<commit_message>
HRS: fix powerlifter widening — every tier must beat other pathways
The prior widening (ratio-scaling every lift from a hand-designed squat
ladder) overcorrected: Beginner/Novice, and for bench/press even Good/
Intermediate, had dropped BELOW every other pathway's corresponding
tier. Redone per-lift instead of by ratio: every tier is hand-picked to
clear the max across all other pathways at that same tier (verified
programmatically against the live generated data). Elite stays exactly
as researched; vestigial `excellent` recomputed as the good/intermediate
midpoint so the browse-standards table stays visually ordered.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -9364,22 +9364,22 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="G75" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="H75" t="n">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="I75" t="n">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="J75" t="n">
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="K75" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="L75" t="n">
         <v>340</v>
@@ -9416,22 +9416,22 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="G76" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H76" t="n">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="I76" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="J76" t="n">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="K76" t="n">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="L76" t="n">
         <v>210</v>
@@ -9468,22 +9468,22 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="G77" t="n">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="H77" t="n">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="I77" t="n">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="J77" t="n">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="K77" t="n">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="L77" t="n">
         <v>280</v>
@@ -9520,22 +9520,22 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G78" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="H78" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="I78" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="J78" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="K78" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="L78" t="n">
         <v>172</v>
@@ -9572,22 +9572,22 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>65</v>
+        <v>125</v>
       </c>
       <c r="G79" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="H79" t="n">
-        <v>145</v>
+        <v>195</v>
       </c>
       <c r="I79" t="n">
-        <v>170</v>
+        <v>220</v>
       </c>
       <c r="J79" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="K79" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="L79" t="n">
         <v>380</v>
@@ -9624,19 +9624,19 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G80" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="H80" t="n">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="I80" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="J80" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="K80" t="n">
         <v>195</v>
@@ -9676,22 +9676,22 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="G81" t="n">
-        <v>65</v>
+        <v>105</v>
       </c>
       <c r="H81" t="n">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="I81" t="n">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="J81" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="K81" t="n">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="L81" t="n">
         <v>240</v>
@@ -9728,22 +9728,22 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G82" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H82" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="I82" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="J82" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="K82" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="L82" t="n">
         <v>135</v>
@@ -9780,22 +9780,22 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G83" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="H83" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="I83" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J83" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="K83" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="L83" t="n">
         <v>135</v>
@@ -9832,22 +9832,22 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G84" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H84" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="I84" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="J84" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="K84" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="L84" t="n">
         <v>75</v>

</xml_diff>

<commit_message>
HRS: General/Bodybuilder Beginner-Novice moved in line with hybrid base
Owner: bring these two pathways' Beginner/Novice down a bit to match the
hybrid athlete base. Good/Intermediate/Advanced/Elite unchanged.
Verified the just-fixed powerlifter floor invariant still holds (lowering
these two pathways only makes powerlifter's floor easier to clear, never
harder).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -931,7 +931,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Squat contested in PL; rich by sex/BW/age | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Front squat 1RM | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Bench contested in PL | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Anchor ratio vs bench / bodyweight; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Comp data elite-biased; anchor with coaching ratios | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>As snatch | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
+          <t>Ratio vs clean &amp; jerk; refine from own data | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW) | 2026-07-12: absolute kg (owner: fixed-load sports don't scale with BW)</t>
         </is>
       </c>
     </row>
@@ -5368,10 +5368,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G3" t="n">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="H3" t="n">
         <v>135</v>
@@ -5420,10 +5420,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -5576,10 +5576,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="G7" t="n">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="H7" t="n">
         <v>150</v>
@@ -5628,10 +5628,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="G8" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H8" t="n">
         <v>85</v>
@@ -5732,10 +5732,10 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G10" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H10" t="n">
         <v>50</v>
@@ -5784,10 +5784,10 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G11" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H11" t="n">
         <v>65</v>
@@ -5888,10 +5888,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" t="n">
         <v>50</v>
-      </c>
-      <c r="G13" t="n">
-        <v>60</v>
       </c>
       <c r="H13" t="n">
         <v>75</v>
@@ -5992,10 +5992,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G15" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H15" t="n">
         <v>90</v>
@@ -6096,10 +6096,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G17" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="H17" t="n">
         <v>90</v>
@@ -6148,10 +6148,10 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G18" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H18" t="n">
         <v>50</v>
@@ -9884,10 +9884,10 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G85" t="n">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="H85" t="n">
         <v>135</v>
@@ -9936,10 +9936,10 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G86" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H86" t="n">
         <v>85</v>
@@ -9991,7 +9991,7 @@
         <v>70</v>
       </c>
       <c r="G87" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H87" t="n">
         <v>110</v>
@@ -10040,10 +10040,10 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G88" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H88" t="n">
         <v>65</v>
@@ -10092,10 +10092,10 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G89" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H89" t="n">
         <v>140</v>
@@ -10248,10 +10248,10 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G92" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H92" t="n">
         <v>53</v>
@@ -10300,7 +10300,7 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G93" t="n">
         <v>50</v>
@@ -10352,10 +10352,10 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G94" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H94" t="n">
         <v>38</v>

</xml_diff>